<commit_message>
Delete duplicates in clean data
</commit_message>
<xml_diff>
--- a/dashboard/jumia_product_dashboard.xlsx
+++ b/dashboard/jumia_product_dashboard.xlsx
@@ -13,7 +13,7 @@
     <sheet name="clean_data" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">clean_data!$A$1:$F$124</definedName>
+    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">clean_data!$A$1:$F$114</definedName>
     <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">raw_data!$A:$I</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
@@ -4382,7 +4382,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F124"/>
+  <dimension ref="A1:F114"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="13.2" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="8" width="68.58"/>
@@ -5535,1925 +5535,1805 @@
     <row r="45" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="8" t="str">
         <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v>Balloon Insert, Birthday Party Balloon Set, Pu Leather</v>
+        <v>Shower Cap Wide Elastic Band Cover Reusable Bashroom Cap</v>
       </c>
       <c r="B45" s="9" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B45), "ksh", ""))), "")</f>
-        <v>610</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B46), "ksh", ""))), "")</f>
+        <v>2132</v>
       </c>
       <c r="C45" s="10" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C45), "ksh", ""))), "")</f>
-        <v>1060</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C46), "ksh", ""))), "")</f>
+        <v>2169</v>
       </c>
       <c r="D45" s="21" t="n">
-        <f aca="false">VALUE(TRIM(raw_data!D45))</f>
-        <v>0.42</v>
+        <f aca="false">VALUE(TRIM(raw_data!D46))</f>
+        <v>0.02</v>
       </c>
       <c r="E45" s="12" t="str">
-        <f aca="false">IF(ISBLANK(raw_data!E45),"",ABS(TRIM(raw_data!E45)))</f>
+        <f aca="false">IF(ISBLANK(raw_data!E46),"",ABS(TRIM(raw_data!E46)))</f>
         <v/>
       </c>
       <c r="F45" s="13" t="str">
-        <f aca="false">=IF(ISBLANK(raw_data!F45),"",VALUE(LEFT(raw_data!F45,FIND(" ", raw_data!F45,1))))</f>
+        <f aca="false">=IF(ISBLANK(raw_data!F46),"",VALUE(LEFT(raw_data!F46,FIND(" ", raw_data!F46,1))))</f>
         <v/>
       </c>
     </row>
     <row r="46" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="8" t="str">
         <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v>Shower Cap Wide Elastic Band Cover Reusable Bashroom Cap</v>
+        <v>Christmas Elk Fence Yard Lawn Decorations Cute For Holidays</v>
       </c>
       <c r="B46" s="9" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B46), "ksh", ""))), "")</f>
-        <v>2132</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B47), "ksh", ""))), "")</f>
+        <v>999</v>
       </c>
       <c r="C46" s="10" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C46), "ksh", ""))), "")</f>
-        <v>2169</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C47), "ksh", ""))), "")</f>
+        <v>2000</v>
       </c>
       <c r="D46" s="21" t="n">
-        <f aca="false">VALUE(TRIM(raw_data!D46))</f>
-        <v>0.02</v>
+        <f aca="false">VALUE(TRIM(raw_data!D47))</f>
+        <v>0.5</v>
       </c>
       <c r="E46" s="12" t="str">
-        <f aca="false">IF(ISBLANK(raw_data!E46),"",ABS(TRIM(raw_data!E46)))</f>
+        <f aca="false">IF(ISBLANK(raw_data!E47),"",ABS(TRIM(raw_data!E47)))</f>
         <v/>
       </c>
       <c r="F46" s="13" t="str">
-        <f aca="false">=IF(ISBLANK(raw_data!F46),"",VALUE(LEFT(raw_data!F46,FIND(" ", raw_data!F46,1))))</f>
+        <f aca="false">=IF(ISBLANK(raw_data!F47),"",VALUE(LEFT(raw_data!F47,FIND(" ", raw_data!F47,1))))</f>
         <v/>
       </c>
     </row>
     <row r="47" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="8" t="str">
         <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v>Christmas Elk Fence Yard Lawn Decorations Cute For Holidays</v>
+        <v>60W Hot Melt Glue Sprayer - Efficient And Stable Glue Dispensing</v>
       </c>
       <c r="B47" s="9" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B47), "ksh", ""))), "")</f>
-        <v>999</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B48), "ksh", ""))), "")</f>
+        <v>1190</v>
       </c>
       <c r="C47" s="10" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C47), "ksh", ""))), "")</f>
-        <v>2000</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C48), "ksh", ""))), "")</f>
+        <v>1785</v>
       </c>
       <c r="D47" s="21" t="n">
-        <f aca="false">VALUE(TRIM(raw_data!D47))</f>
-        <v>0.5</v>
+        <f aca="false">VALUE(TRIM(raw_data!D48))</f>
+        <v>0.33</v>
       </c>
       <c r="E47" s="12" t="str">
-        <f aca="false">IF(ISBLANK(raw_data!E47),"",ABS(TRIM(raw_data!E47)))</f>
+        <f aca="false">IF(ISBLANK(raw_data!E48),"",ABS(TRIM(raw_data!E48)))</f>
         <v/>
       </c>
       <c r="F47" s="13" t="str">
-        <f aca="false">=IF(ISBLANK(raw_data!F47),"",VALUE(LEFT(raw_data!F47,FIND(" ", raw_data!F47,1))))</f>
+        <f aca="false">=IF(ISBLANK(raw_data!F48),"",VALUE(LEFT(raw_data!F48,FIND(" ", raw_data!F48,1))))</f>
         <v/>
       </c>
     </row>
     <row r="48" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="8" t="str">
         <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v>60W Hot Melt Glue Sprayer - Efficient And Stable Glue Dispensing</v>
+        <v>Car Phone Charging Stand</v>
       </c>
       <c r="B48" s="9" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B48), "ksh", ""))), "")</f>
-        <v>1190</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B49), "ksh", ""))), "")</f>
+        <v>671</v>
       </c>
       <c r="C48" s="10" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C48), "ksh", ""))), "")</f>
-        <v>1785</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C49), "ksh", ""))), "")</f>
+        <v>1316</v>
       </c>
       <c r="D48" s="21" t="n">
-        <f aca="false">VALUE(TRIM(raw_data!D48))</f>
-        <v>0.33</v>
+        <f aca="false">VALUE(TRIM(raw_data!D49))</f>
+        <v>0.49</v>
       </c>
       <c r="E48" s="12" t="str">
-        <f aca="false">IF(ISBLANK(raw_data!E48),"",ABS(TRIM(raw_data!E48)))</f>
+        <f aca="false">IF(ISBLANK(raw_data!E49),"",ABS(TRIM(raw_data!E49)))</f>
         <v/>
       </c>
       <c r="F48" s="13" t="str">
-        <f aca="false">=IF(ISBLANK(raw_data!F48),"",VALUE(LEFT(raw_data!F48,FIND(" ", raw_data!F48,1))))</f>
+        <f aca="false">=IF(ISBLANK(raw_data!F49),"",VALUE(LEFT(raw_data!F49,FIND(" ", raw_data!F49,1))))</f>
         <v/>
       </c>
     </row>
     <row r="49" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="8" t="str">
         <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v>Car Phone Charging Stand</v>
+        <v>2Pcs Solar Street Light Flood Light Outdoor</v>
       </c>
       <c r="B49" s="9" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B49), "ksh", ""))), "")</f>
-        <v>671</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B50), "ksh", ""))), "")</f>
+        <v>1200</v>
       </c>
       <c r="C49" s="10" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C49), "ksh", ""))), "")</f>
-        <v>1316</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C50), "ksh", ""))), "")</f>
+        <v>1950</v>
       </c>
       <c r="D49" s="21" t="n">
-        <f aca="false">VALUE(TRIM(raw_data!D49))</f>
-        <v>0.49</v>
+        <f aca="false">VALUE(TRIM(raw_data!D50))</f>
+        <v>0.38</v>
       </c>
       <c r="E49" s="12" t="str">
-        <f aca="false">IF(ISBLANK(raw_data!E49),"",ABS(TRIM(raw_data!E49)))</f>
+        <f aca="false">IF(ISBLANK(raw_data!E50),"",ABS(TRIM(raw_data!E50)))</f>
         <v/>
       </c>
       <c r="F49" s="13" t="str">
-        <f aca="false">=IF(ISBLANK(raw_data!F49),"",VALUE(LEFT(raw_data!F49,FIND(" ", raw_data!F49,1))))</f>
+        <f aca="false">=IF(ISBLANK(raw_data!F50),"",VALUE(LEFT(raw_data!F50,FIND(" ", raw_data!F50,1))))</f>
         <v/>
       </c>
     </row>
     <row r="50" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="8" t="str">
         <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v>2Pcs Solar Street Light Flood Light Outdoor</v>
+        <v>Creative Owl Shape Keychain Black</v>
       </c>
       <c r="B50" s="9" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B50), "ksh", ""))), "")</f>
-        <v>1200</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B51), "ksh", ""))), "")</f>
+        <v>199</v>
       </c>
       <c r="C50" s="10" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C50), "ksh", ""))), "")</f>
-        <v>1950</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C51), "ksh", ""))), "")</f>
+        <v>504</v>
       </c>
       <c r="D50" s="21" t="n">
-        <f aca="false">VALUE(TRIM(raw_data!D50))</f>
-        <v>0.38</v>
+        <f aca="false">VALUE(TRIM(raw_data!D51))</f>
+        <v>0.61</v>
       </c>
       <c r="E50" s="12" t="str">
-        <f aca="false">IF(ISBLANK(raw_data!E50),"",ABS(TRIM(raw_data!E50)))</f>
+        <f aca="false">IF(ISBLANK(raw_data!E51),"",ABS(TRIM(raw_data!E51)))</f>
         <v/>
       </c>
       <c r="F50" s="13" t="str">
-        <f aca="false">=IF(ISBLANK(raw_data!F50),"",VALUE(LEFT(raw_data!F50,FIND(" ", raw_data!F50,1))))</f>
+        <f aca="false">=IF(ISBLANK(raw_data!F51),"",VALUE(LEFT(raw_data!F51,FIND(" ", raw_data!F51,1))))</f>
         <v/>
       </c>
     </row>
     <row r="51" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="8" t="str">
         <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v>Creative Owl Shape Keychain Black</v>
+        <v>Brush &amp; Paintbrush Cleaning Tool Pink</v>
       </c>
       <c r="B51" s="9" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B51), "ksh", ""))), "")</f>
-        <v>199</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B52), "ksh", ""))), "")</f>
+        <v>299</v>
       </c>
       <c r="C51" s="10" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C51), "ksh", ""))), "")</f>
-        <v>504</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C52), "ksh", ""))), "")</f>
+        <v>600</v>
       </c>
       <c r="D51" s="21" t="n">
-        <f aca="false">VALUE(TRIM(raw_data!D51))</f>
-        <v>0.61</v>
+        <f aca="false">VALUE(TRIM(raw_data!D52))</f>
+        <v>0.5</v>
       </c>
       <c r="E51" s="12" t="str">
-        <f aca="false">IF(ISBLANK(raw_data!E51),"",ABS(TRIM(raw_data!E51)))</f>
+        <f aca="false">IF(ISBLANK(raw_data!E52),"",ABS(TRIM(raw_data!E52)))</f>
         <v/>
       </c>
       <c r="F51" s="13" t="str">
-        <f aca="false">=IF(ISBLANK(raw_data!F51),"",VALUE(LEFT(raw_data!F51,FIND(" ", raw_data!F51,1))))</f>
+        <f aca="false">=IF(ISBLANK(raw_data!F52),"",VALUE(LEFT(raw_data!F52,FIND(" ", raw_data!F52,1))))</f>
         <v/>
       </c>
     </row>
     <row r="52" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="8" t="str">
         <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v>Brush &amp; Paintbrush Cleaning Tool Pink</v>
+        <v>Pen Grips For Kids Pen Grip Posture Correction Tool For Kids</v>
       </c>
       <c r="B52" s="9" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B52), "ksh", ""))), "")</f>
-        <v>299</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B53), "ksh", ""))), "")</f>
+        <v>1660</v>
       </c>
       <c r="C52" s="10" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C52), "ksh", ""))), "")</f>
-        <v>600</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C53), "ksh", ""))), "")</f>
+        <v>1699</v>
       </c>
       <c r="D52" s="21" t="n">
-        <f aca="false">VALUE(TRIM(raw_data!D52))</f>
-        <v>0.5</v>
+        <f aca="false">VALUE(TRIM(raw_data!D53))</f>
+        <v>0.02</v>
       </c>
       <c r="E52" s="12" t="str">
-        <f aca="false">IF(ISBLANK(raw_data!E52),"",ABS(TRIM(raw_data!E52)))</f>
+        <f aca="false">IF(ISBLANK(raw_data!E53),"",ABS(TRIM(raw_data!E53)))</f>
         <v/>
       </c>
       <c r="F52" s="13" t="str">
-        <f aca="false">=IF(ISBLANK(raw_data!F52),"",VALUE(LEFT(raw_data!F52,FIND(" ", raw_data!F52,1))))</f>
+        <f aca="false">=IF(ISBLANK(raw_data!F53),"",VALUE(LEFT(raw_data!F53,FIND(" ", raw_data!F53,1))))</f>
         <v/>
       </c>
     </row>
     <row r="53" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="8" t="str">
         <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v>Pen Grips For Kids Pen Grip Posture Correction Tool For Kids</v>
+        <v>Pilates Cloth Bag Waterproof Durable High Capacity Purple</v>
       </c>
       <c r="B53" s="9" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B53), "ksh", ""))), "")</f>
-        <v>1660</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B54), "ksh", ""))), "")</f>
+        <v>299</v>
       </c>
       <c r="C53" s="10" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C53), "ksh", ""))), "")</f>
-        <v>1699</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C54), "ksh", ""))), "")</f>
+        <v>384</v>
       </c>
       <c r="D53" s="21" t="n">
-        <f aca="false">VALUE(TRIM(raw_data!D53))</f>
-        <v>0.02</v>
+        <f aca="false">VALUE(TRIM(raw_data!D54))</f>
+        <v>0.22</v>
       </c>
       <c r="E53" s="12" t="str">
-        <f aca="false">IF(ISBLANK(raw_data!E53),"",ABS(TRIM(raw_data!E53)))</f>
+        <f aca="false">IF(ISBLANK(raw_data!E54),"",ABS(TRIM(raw_data!E54)))</f>
         <v/>
       </c>
       <c r="F53" s="13" t="str">
-        <f aca="false">=IF(ISBLANK(raw_data!F53),"",VALUE(LEFT(raw_data!F53,FIND(" ", raw_data!F53,1))))</f>
+        <f aca="false">=IF(ISBLANK(raw_data!F54),"",VALUE(LEFT(raw_data!F54,FIND(" ", raw_data!F54,1))))</f>
         <v/>
       </c>
     </row>
     <row r="54" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="8" t="str">
         <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v>Pilates Cloth Bag Waterproof Durable High Capacity Purple</v>
+        <v>Multi-Purpose Rice Drainage Basket And Fruit And Vegetable Drainage Sieve</v>
       </c>
       <c r="B54" s="9" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B54), "ksh", ""))), "")</f>
-        <v>299</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B55), "ksh", ""))), "")</f>
+        <v>1459</v>
       </c>
       <c r="C54" s="10" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C54), "ksh", ""))), "")</f>
-        <v>384</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C55), "ksh", ""))), "")</f>
+        <v>1499</v>
       </c>
       <c r="D54" s="21" t="n">
-        <f aca="false">VALUE(TRIM(raw_data!D54))</f>
-        <v>0.22</v>
+        <f aca="false">VALUE(TRIM(raw_data!D55))</f>
+        <v>0.03</v>
       </c>
       <c r="E54" s="12" t="str">
-        <f aca="false">IF(ISBLANK(raw_data!E54),"",ABS(TRIM(raw_data!E54)))</f>
+        <f aca="false">IF(ISBLANK(raw_data!E55),"",ABS(TRIM(raw_data!E55)))</f>
         <v/>
       </c>
       <c r="F54" s="13" t="str">
-        <f aca="false">=IF(ISBLANK(raw_data!F54),"",VALUE(LEFT(raw_data!F54,FIND(" ", raw_data!F54,1))))</f>
+        <f aca="false">=IF(ISBLANK(raw_data!F55),"",VALUE(LEFT(raw_data!F55,FIND(" ", raw_data!F55,1))))</f>
         <v/>
       </c>
     </row>
     <row r="55" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="8" t="str">
         <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v>Multi-Purpose Rice Drainage Basket And Fruit And Vegetable Drainage Sieve</v>
+        <v>Cute Christmas Fence Garden Decorations For Holiday Home</v>
       </c>
       <c r="B55" s="9" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B55), "ksh", ""))), "")</f>
-        <v>1459</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B56), "ksh", ""))), "")</f>
+        <v>799</v>
       </c>
       <c r="C55" s="10" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C55), "ksh", ""))), "")</f>
-        <v>1499</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C56), "ksh", ""))), "")</f>
+        <v>1343</v>
       </c>
       <c r="D55" s="21" t="n">
-        <f aca="false">VALUE(TRIM(raw_data!D55))</f>
-        <v>0.03</v>
+        <f aca="false">VALUE(TRIM(raw_data!D56))</f>
+        <v>0.41</v>
       </c>
       <c r="E55" s="12" t="str">
-        <f aca="false">IF(ISBLANK(raw_data!E55),"",ABS(TRIM(raw_data!E55)))</f>
+        <f aca="false">IF(ISBLANK(raw_data!E56),"",ABS(TRIM(raw_data!E56)))</f>
         <v/>
       </c>
       <c r="F55" s="13" t="str">
-        <f aca="false">=IF(ISBLANK(raw_data!F55),"",VALUE(LEFT(raw_data!F55,FIND(" ", raw_data!F55,1))))</f>
+        <f aca="false">=IF(ISBLANK(raw_data!F56),"",VALUE(LEFT(raw_data!F56,FIND(" ", raw_data!F56,1))))</f>
         <v/>
       </c>
     </row>
     <row r="56" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="8" t="str">
         <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v>Cute Christmas Fence Garden Decorations For Holiday Home</v>
+        <v>Simple Metal Dog Art Sculpture Decoration For Home Office</v>
       </c>
       <c r="B56" s="9" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B56), "ksh", ""))), "")</f>
-        <v>799</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B57), "ksh", ""))), "")</f>
+        <v>499</v>
       </c>
       <c r="C56" s="10" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C56), "ksh", ""))), "")</f>
-        <v>1343</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C57), "ksh", ""))), "")</f>
+        <v>900</v>
       </c>
       <c r="D56" s="21" t="n">
-        <f aca="false">VALUE(TRIM(raw_data!D56))</f>
-        <v>0.41</v>
+        <f aca="false">VALUE(TRIM(raw_data!D57))</f>
+        <v>0.45</v>
       </c>
       <c r="E56" s="12" t="str">
-        <f aca="false">IF(ISBLANK(raw_data!E56),"",ABS(TRIM(raw_data!E56)))</f>
+        <f aca="false">IF(ISBLANK(raw_data!E57),"",ABS(TRIM(raw_data!E57)))</f>
         <v/>
       </c>
       <c r="F56" s="13" t="str">
-        <f aca="false">=IF(ISBLANK(raw_data!F56),"",VALUE(LEFT(raw_data!F56,FIND(" ", raw_data!F56,1))))</f>
+        <f aca="false">=IF(ISBLANK(raw_data!F57),"",VALUE(LEFT(raw_data!F57,FIND(" ", raw_data!F57,1))))</f>
         <v/>
       </c>
     </row>
     <row r="57" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="8" t="str">
         <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v>Simple Metal Dog Art Sculpture Decoration For Home Office</v>
+        <v>Christmas Fence Garden Decorations Outdoor For Holiday Home</v>
       </c>
       <c r="B57" s="9" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B57), "ksh", ""))), "")</f>
-        <v>499</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B58), "ksh", ""))), "")</f>
+        <v>699</v>
       </c>
       <c r="C57" s="10" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C57), "ksh", ""))), "")</f>
-        <v>900</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C58), "ksh", ""))), "")</f>
+        <v>1343</v>
       </c>
       <c r="D57" s="21" t="n">
-        <f aca="false">VALUE(TRIM(raw_data!D57))</f>
-        <v>0.45</v>
+        <f aca="false">VALUE(TRIM(raw_data!D58))</f>
+        <v>0.48</v>
       </c>
       <c r="E57" s="12" t="str">
-        <f aca="false">IF(ISBLANK(raw_data!E57),"",ABS(TRIM(raw_data!E57)))</f>
+        <f aca="false">IF(ISBLANK(raw_data!E58),"",ABS(TRIM(raw_data!E58)))</f>
         <v/>
       </c>
       <c r="F57" s="13" t="str">
-        <f aca="false">=IF(ISBLANK(raw_data!F57),"",VALUE(LEFT(raw_data!F57,FIND(" ", raw_data!F57,1))))</f>
+        <f aca="false">=IF(ISBLANK(raw_data!F58),"",VALUE(LEFT(raw_data!F58,FIND(" ", raw_data!F58,1))))</f>
         <v/>
       </c>
     </row>
     <row r="58" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="8" t="str">
         <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v>Christmas Fence Garden Decorations Outdoor For Holiday Home</v>
+        <v>Angle Measuring Tool Full Metal Multi Angle Measuring Tool</v>
       </c>
       <c r="B58" s="9" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B58), "ksh", ""))), "")</f>
-        <v>699</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B59), "ksh", ""))), "")</f>
+        <v>799</v>
       </c>
       <c r="C58" s="10" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C58), "ksh", ""))), "")</f>
-        <v>1343</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C59), "ksh", ""))), "")</f>
+        <v>1567</v>
       </c>
       <c r="D58" s="21" t="n">
-        <f aca="false">VALUE(TRIM(raw_data!D58))</f>
-        <v>0.48</v>
+        <f aca="false">VALUE(TRIM(raw_data!D59))</f>
+        <v>0.49</v>
       </c>
       <c r="E58" s="12" t="str">
-        <f aca="false">IF(ISBLANK(raw_data!E58),"",ABS(TRIM(raw_data!E58)))</f>
+        <f aca="false">IF(ISBLANK(raw_data!E59),"",ABS(TRIM(raw_data!E59)))</f>
         <v/>
       </c>
       <c r="F58" s="13" t="str">
-        <f aca="false">=IF(ISBLANK(raw_data!F58),"",VALUE(LEFT(raw_data!F58,FIND(" ", raw_data!F58,1))))</f>
+        <f aca="false">=IF(ISBLANK(raw_data!F59),"",VALUE(LEFT(raw_data!F59,FIND(" ", raw_data!F59,1))))</f>
         <v/>
       </c>
     </row>
     <row r="59" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="8" t="str">
         <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v>Angle Measuring Tool Full Metal Multi Angle Measuring Tool</v>
+        <v>12V 19500Rpm Handheld Electric Angle Grinder Tool - Uk - Yellow/Black</v>
       </c>
       <c r="B59" s="9" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B59), "ksh", ""))), "")</f>
-        <v>799</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B60), "ksh", ""))), "")</f>
+        <v>2799</v>
       </c>
       <c r="C59" s="10" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C59), "ksh", ""))), "")</f>
-        <v>1567</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C60), "ksh", ""))), "")</f>
+        <v>3810</v>
       </c>
       <c r="D59" s="21" t="n">
-        <f aca="false">VALUE(TRIM(raw_data!D59))</f>
-        <v>0.49</v>
+        <f aca="false">VALUE(TRIM(raw_data!D60))</f>
+        <v>0.27</v>
       </c>
       <c r="E59" s="12" t="str">
-        <f aca="false">IF(ISBLANK(raw_data!E59),"",ABS(TRIM(raw_data!E59)))</f>
+        <f aca="false">IF(ISBLANK(raw_data!E60),"",ABS(TRIM(raw_data!E60)))</f>
         <v/>
       </c>
       <c r="F59" s="13" t="str">
-        <f aca="false">=IF(ISBLANK(raw_data!F59),"",VALUE(LEFT(raw_data!F59,FIND(" ", raw_data!F59,1))))</f>
+        <f aca="false">=IF(ISBLANK(raw_data!F60),"",VALUE(LEFT(raw_data!F60,FIND(" ", raw_data!F60,1))))</f>
         <v/>
       </c>
     </row>
     <row r="60" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="8" t="str">
         <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v>12V 19500Rpm Handheld Electric Angle Grinder Tool - Uk - Yellow/Black</v>
+        <v>Simple Metal Dog Art Sculpture Decoration For Home Office</v>
       </c>
       <c r="B60" s="9" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B60), "ksh", ""))), "")</f>
-        <v>2799</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B61), "ksh", ""))), "")</f>
+        <v>399</v>
       </c>
       <c r="C60" s="10" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C60), "ksh", ""))), "")</f>
-        <v>3810</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C61), "ksh", ""))), "")</f>
+        <v>896</v>
       </c>
       <c r="D60" s="21" t="n">
-        <f aca="false">VALUE(TRIM(raw_data!D60))</f>
-        <v>0.27</v>
+        <f aca="false">VALUE(TRIM(raw_data!D61))</f>
+        <v>0.55</v>
       </c>
       <c r="E60" s="12" t="str">
-        <f aca="false">IF(ISBLANK(raw_data!E60),"",ABS(TRIM(raw_data!E60)))</f>
+        <f aca="false">IF(ISBLANK(raw_data!E61),"",ABS(TRIM(raw_data!E61)))</f>
         <v/>
       </c>
       <c r="F60" s="13" t="str">
-        <f aca="false">=IF(ISBLANK(raw_data!F60),"",VALUE(LEFT(raw_data!F60,FIND(" ", raw_data!F60,1))))</f>
+        <f aca="false">=IF(ISBLANK(raw_data!F61),"",VALUE(LEFT(raw_data!F61,FIND(" ", raw_data!F61,1))))</f>
         <v/>
       </c>
     </row>
     <row r="61" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="8" t="str">
         <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v>Simple Metal Dog Art Sculpture Decoration For Home Office</v>
+        <v>5 Pieces/Set Of Stainless Steel Induction Cooker Pots</v>
       </c>
       <c r="B61" s="9" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B61), "ksh", ""))), "")</f>
-        <v>399</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B62), "ksh", ""))), "")</f>
+        <v>2170</v>
       </c>
       <c r="C61" s="10" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C61), "ksh", ""))), "")</f>
-        <v>896</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C62), "ksh", ""))), "")</f>
+        <v>2500</v>
       </c>
       <c r="D61" s="21" t="n">
-        <f aca="false">VALUE(TRIM(raw_data!D61))</f>
-        <v>0.55</v>
-      </c>
-      <c r="E61" s="12" t="str">
-        <f aca="false">IF(ISBLANK(raw_data!E61),"",ABS(TRIM(raw_data!E61)))</f>
-        <v/>
-      </c>
-      <c r="F61" s="13" t="str">
-        <f aca="false">=IF(ISBLANK(raw_data!F61),"",VALUE(LEFT(raw_data!F61,FIND(" ", raw_data!F61,1))))</f>
-        <v/>
+        <f aca="false">VALUE(TRIM(raw_data!D62))</f>
+        <v>0.13</v>
+      </c>
+      <c r="E61" s="12" t="n">
+        <f aca="false">IF(ISBLANK(raw_data!E62),"",ABS(TRIM(raw_data!E62)))</f>
+        <v>6</v>
+      </c>
+      <c r="F61" s="13" t="n">
+        <f aca="false">=IF(ISBLANK(raw_data!F62),"",VALUE(LEFT(raw_data!F62,FIND(" ", raw_data!F62,1))))</f>
+        <v>2.5</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="8" t="str">
         <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v>5 Pieces/Set Of Stainless Steel Induction Cooker Pots</v>
+        <v>Mythco 120Cob Solar Wall Ligt With Motion Sensor And Remote Control 3 Modes</v>
       </c>
       <c r="B62" s="9" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B62), "ksh", ""))), "")</f>
-        <v>2170</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B63), "ksh", ""))), "")</f>
+        <v>458</v>
       </c>
       <c r="C62" s="10" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C62), "ksh", ""))), "")</f>
-        <v>2500</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C63), "ksh", ""))), "")</f>
+        <v>986</v>
       </c>
       <c r="D62" s="21" t="n">
-        <f aca="false">VALUE(TRIM(raw_data!D62))</f>
-        <v>0.13</v>
+        <f aca="false">VALUE(TRIM(raw_data!D63))</f>
+        <v>0.54</v>
       </c>
       <c r="E62" s="12" t="n">
-        <f aca="false">IF(ISBLANK(raw_data!E62),"",ABS(TRIM(raw_data!E62)))</f>
-        <v>6</v>
+        <f aca="false">IF(ISBLANK(raw_data!E63),"",ABS(TRIM(raw_data!E63)))</f>
+        <v>10</v>
       </c>
       <c r="F62" s="13" t="n">
-        <f aca="false">=IF(ISBLANK(raw_data!F62),"",VALUE(LEFT(raw_data!F62,FIND(" ", raw_data!F62,1))))</f>
-        <v>2.5</v>
+        <f aca="false">=IF(ISBLANK(raw_data!F63),"",VALUE(LEFT(raw_data!F63,FIND(" ", raw_data!F63,1))))</f>
+        <v>3</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="8" t="str">
         <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v>Mythco 120Cob Solar Wall Ligt With Motion Sensor And Remote Control 3 Modes</v>
+        <v>5-Pcs Stainless Steel Cooking Pot Set With Steamed Slices</v>
       </c>
       <c r="B63" s="9" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B63), "ksh", ""))), "")</f>
-        <v>458</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B64), "ksh", ""))), "")</f>
+        <v>2115</v>
       </c>
       <c r="C63" s="10" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C63), "ksh", ""))), "")</f>
-        <v>986</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C64), "ksh", ""))), "")</f>
+        <v>4700</v>
       </c>
       <c r="D63" s="21" t="n">
-        <f aca="false">VALUE(TRIM(raw_data!D63))</f>
-        <v>0.54</v>
+        <f aca="false">VALUE(TRIM(raw_data!D64))</f>
+        <v>0.55</v>
       </c>
       <c r="E63" s="12" t="n">
-        <f aca="false">IF(ISBLANK(raw_data!E63),"",ABS(TRIM(raw_data!E63)))</f>
-        <v>10</v>
+        <f aca="false">IF(ISBLANK(raw_data!E64),"",ABS(TRIM(raw_data!E64)))</f>
+        <v>13</v>
       </c>
       <c r="F63" s="13" t="n">
-        <f aca="false">=IF(ISBLANK(raw_data!F63),"",VALUE(LEFT(raw_data!F63,FIND(" ", raw_data!F63,1))))</f>
-        <v>3</v>
+        <f aca="false">=IF(ISBLANK(raw_data!F64),"",VALUE(LEFT(raw_data!F64,FIND(" ", raw_data!F64,1))))</f>
+        <v>2.1</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="8" t="str">
         <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v>5-Pcs Stainless Steel Cooking Pot Set With Steamed Slices</v>
+        <v>120W Cordless Vacuum Cleaners Handheld Electric Vacuum Cleaner</v>
       </c>
       <c r="B64" s="9" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B64), "ksh", ""))), "")</f>
-        <v>2115</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B65), "ksh", ""))), "")</f>
+        <v>445</v>
       </c>
       <c r="C64" s="10" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C64), "ksh", ""))), "")</f>
-        <v>4700</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C65), "ksh", ""))), "")</f>
+        <v>873</v>
       </c>
       <c r="D64" s="21" t="n">
-        <f aca="false">VALUE(TRIM(raw_data!D64))</f>
-        <v>0.55</v>
+        <f aca="false">VALUE(TRIM(raw_data!D65))</f>
+        <v>0.49</v>
       </c>
       <c r="E64" s="12" t="n">
-        <f aca="false">IF(ISBLANK(raw_data!E64),"",ABS(TRIM(raw_data!E64)))</f>
-        <v>13</v>
+        <f aca="false">IF(ISBLANK(raw_data!E65),"",ABS(TRIM(raw_data!E65)))</f>
+        <v>69</v>
       </c>
       <c r="F64" s="13" t="n">
-        <f aca="false">=IF(ISBLANK(raw_data!F64),"",VALUE(LEFT(raw_data!F64,FIND(" ", raw_data!F64,1))))</f>
-        <v>2.1</v>
+        <f aca="false">=IF(ISBLANK(raw_data!F65),"",VALUE(LEFT(raw_data!F65,FIND(" ", raw_data!F65,1))))</f>
+        <v>2.8</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="8" t="str">
         <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v>120W Cordless Vacuum Cleaners Handheld Electric Vacuum Cleaner</v>
+        <v>Intelligent Led Body Sensor Wireless Lighting Night Light Usb</v>
       </c>
       <c r="B65" s="9" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B65), "ksh", ""))), "")</f>
-        <v>445</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B66), "ksh", ""))), "")</f>
+        <v>325</v>
       </c>
       <c r="C65" s="10" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C65), "ksh", ""))), "")</f>
-        <v>873</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C66), "ksh", ""))), "")</f>
+        <v>680</v>
       </c>
       <c r="D65" s="21" t="n">
-        <f aca="false">VALUE(TRIM(raw_data!D65))</f>
-        <v>0.49</v>
+        <f aca="false">VALUE(TRIM(raw_data!D66))</f>
+        <v>0.52</v>
       </c>
       <c r="E65" s="12" t="n">
-        <f aca="false">IF(ISBLANK(raw_data!E65),"",ABS(TRIM(raw_data!E65)))</f>
-        <v>69</v>
+        <f aca="false">IF(ISBLANK(raw_data!E66),"",ABS(TRIM(raw_data!E66)))</f>
+        <v>15</v>
       </c>
       <c r="F65" s="13" t="n">
-        <f aca="false">=IF(ISBLANK(raw_data!F65),"",VALUE(LEFT(raw_data!F65,FIND(" ", raw_data!F65,1))))</f>
-        <v>2.8</v>
+        <f aca="false">=IF(ISBLANK(raw_data!F66),"",VALUE(LEFT(raw_data!F66,FIND(" ", raw_data!F66,1))))</f>
+        <v>2.7</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="8" t="str">
         <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v>Intelligent Led Body Sensor Wireless Lighting Night Light Usb</v>
+        <v>Vic Wireless Vacuum Cleaner Dual Use For Home And Car 120W High Power Powerful</v>
       </c>
       <c r="B66" s="9" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B66), "ksh", ""))), "")</f>
-        <v>325</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B67), "ksh", ""))), "")</f>
+        <v>1220</v>
       </c>
       <c r="C66" s="10" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C66), "ksh", ""))), "")</f>
-        <v>680</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C67), "ksh", ""))), "")</f>
+        <v>1555</v>
       </c>
       <c r="D66" s="21" t="n">
-        <f aca="false">VALUE(TRIM(raw_data!D66))</f>
-        <v>0.52</v>
+        <f aca="false">VALUE(TRIM(raw_data!D67))</f>
+        <v>0.22</v>
       </c>
       <c r="E66" s="12" t="n">
-        <f aca="false">IF(ISBLANK(raw_data!E66),"",ABS(TRIM(raw_data!E66)))</f>
-        <v>15</v>
+        <f aca="false">IF(ISBLANK(raw_data!E67),"",ABS(TRIM(raw_data!E67)))</f>
+        <v>16</v>
       </c>
       <c r="F66" s="13" t="n">
-        <f aca="false">=IF(ISBLANK(raw_data!F66),"",VALUE(LEFT(raw_data!F66,FIND(" ", raw_data!F66,1))))</f>
-        <v>2.7</v>
+        <f aca="false">=IF(ISBLANK(raw_data!F67),"",VALUE(LEFT(raw_data!F67,FIND(" ", raw_data!F67,1))))</f>
+        <v>2.9</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="8" t="str">
         <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v>Vic Wireless Vacuum Cleaner Dual Use For Home And Car 120W High Power Powerful</v>
+        <v>Artificial Potted Flowers Room Decorative Flowers (2 Pieces)</v>
       </c>
       <c r="B67" s="9" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B67), "ksh", ""))), "")</f>
-        <v>1220</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B68), "ksh", ""))), "")</f>
+        <v>990</v>
       </c>
       <c r="C67" s="10" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C67), "ksh", ""))), "")</f>
-        <v>1555</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C68), "ksh", ""))), "")</f>
+        <v>1814</v>
       </c>
       <c r="D67" s="21" t="n">
-        <f aca="false">VALUE(TRIM(raw_data!D67))</f>
-        <v>0.22</v>
+        <f aca="false">VALUE(TRIM(raw_data!D68))</f>
+        <v>0.45</v>
       </c>
       <c r="E67" s="12" t="n">
-        <f aca="false">IF(ISBLANK(raw_data!E67),"",ABS(TRIM(raw_data!E67)))</f>
-        <v>16</v>
+        <f aca="false">IF(ISBLANK(raw_data!E68),"",ABS(TRIM(raw_data!E68)))</f>
+        <v>6</v>
       </c>
       <c r="F67" s="13" t="n">
-        <f aca="false">=IF(ISBLANK(raw_data!F67),"",VALUE(LEFT(raw_data!F67,FIND(" ", raw_data!F67,1))))</f>
-        <v>2.9</v>
+        <f aca="false">=IF(ISBLANK(raw_data!F68),"",VALUE(LEFT(raw_data!F68,FIND(" ", raw_data!F68,1))))</f>
+        <v>2.2</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="8" t="str">
         <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v>Artificial Potted Flowers Room Decorative Flowers (2 Pieces)</v>
+        <v>380Ml Usb Rechargeable Portable Small Blenders And Juicers</v>
       </c>
       <c r="B68" s="9" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B68), "ksh", ""))), "")</f>
-        <v>990</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B69), "ksh", ""))), "")</f>
+        <v>1000</v>
       </c>
       <c r="C68" s="10" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C68), "ksh", ""))), "")</f>
-        <v>1814</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C69), "ksh", ""))), "")</f>
+        <v>2000</v>
       </c>
       <c r="D68" s="21" t="n">
-        <f aca="false">VALUE(TRIM(raw_data!D68))</f>
-        <v>0.45</v>
+        <f aca="false">VALUE(TRIM(raw_data!D69))</f>
+        <v>0.5</v>
       </c>
       <c r="E68" s="12" t="n">
-        <f aca="false">IF(ISBLANK(raw_data!E68),"",ABS(TRIM(raw_data!E68)))</f>
-        <v>6</v>
+        <f aca="false">IF(ISBLANK(raw_data!E69),"",ABS(TRIM(raw_data!E69)))</f>
+        <v>7</v>
       </c>
       <c r="F68" s="13" t="n">
-        <f aca="false">=IF(ISBLANK(raw_data!F68),"",VALUE(LEFT(raw_data!F68,FIND(" ", raw_data!F68,1))))</f>
-        <v>2.2</v>
+        <f aca="false">=IF(ISBLANK(raw_data!F69),"",VALUE(LEFT(raw_data!F69,FIND(" ", raw_data!F69,1))))</f>
+        <v>2.3</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="8" t="str">
         <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v>380Ml Usb Rechargeable Portable Small Blenders And Juicers</v>
+        <v>32Pcs Portable Cordless Drill Set With Cyclic Battery Drive -26 Variable Speed</v>
       </c>
       <c r="B69" s="9" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B69), "ksh", ""))), "")</f>
-        <v>1000</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B70), "ksh", ""))), "")</f>
+        <v>3750</v>
       </c>
       <c r="C69" s="10" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C69), "ksh", ""))), "")</f>
-        <v>2000</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C70), "ksh", ""))), "")</f>
+        <v>6143</v>
       </c>
       <c r="D69" s="21" t="n">
-        <f aca="false">VALUE(TRIM(raw_data!D69))</f>
-        <v>0.5</v>
+        <f aca="false">VALUE(TRIM(raw_data!D70))</f>
+        <v>0.39</v>
       </c>
       <c r="E69" s="12" t="n">
-        <f aca="false">IF(ISBLANK(raw_data!E69),"",ABS(TRIM(raw_data!E69)))</f>
-        <v>7</v>
+        <f aca="false">IF(ISBLANK(raw_data!E70),"",ABS(TRIM(raw_data!E70)))</f>
+        <v>5</v>
       </c>
       <c r="F69" s="13" t="n">
-        <f aca="false">=IF(ISBLANK(raw_data!F69),"",VALUE(LEFT(raw_data!F69,FIND(" ", raw_data!F69,1))))</f>
-        <v>2.3</v>
+        <f aca="false">=IF(ISBLANK(raw_data!F70),"",VALUE(LEFT(raw_data!F70,FIND(" ", raw_data!F70,1))))</f>
+        <v>3</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="8" t="str">
         <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v>32Pcs Portable Cordless Drill Set With Cyclic Battery Drive -26 Variable Speed</v>
+        <v>Agapeon Toothbrush Holder And Toothpaste Dispenser</v>
       </c>
       <c r="B70" s="9" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B70), "ksh", ""))), "")</f>
-        <v>3750</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B71), "ksh", ""))), "")</f>
+        <v>382</v>
       </c>
       <c r="C70" s="10" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C70), "ksh", ""))), "")</f>
-        <v>6143</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C71), "ksh", ""))), "")</f>
+        <v>700</v>
       </c>
       <c r="D70" s="21" t="n">
-        <f aca="false">VALUE(TRIM(raw_data!D70))</f>
-        <v>0.39</v>
+        <f aca="false">VALUE(TRIM(raw_data!D71))</f>
+        <v>0.45</v>
       </c>
       <c r="E70" s="12" t="n">
-        <f aca="false">IF(ISBLANK(raw_data!E70),"",ABS(TRIM(raw_data!E70)))</f>
-        <v>5</v>
+        <f aca="false">IF(ISBLANK(raw_data!E71),"",ABS(TRIM(raw_data!E71)))</f>
+        <v>17</v>
       </c>
       <c r="F70" s="13" t="n">
-        <f aca="false">=IF(ISBLANK(raw_data!F70),"",VALUE(LEFT(raw_data!F70,FIND(" ", raw_data!F70,1))))</f>
-        <v>3</v>
+        <f aca="false">=IF(ISBLANK(raw_data!F71),"",VALUE(LEFT(raw_data!F71,FIND(" ", raw_data!F71,1))))</f>
+        <v>2.6</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="8" t="str">
         <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v>Agapeon Toothbrush Holder And Toothpaste Dispenser</v>
+        <v>Large Lazy Inflatable Sofa Chairs Pvc Lounger Seat Bag</v>
       </c>
       <c r="B71" s="9" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B71), "ksh", ""))), "")</f>
-        <v>382</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B72), "ksh", ""))), "")</f>
+        <v>2300</v>
       </c>
       <c r="C71" s="10" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C71), "ksh", ""))), "")</f>
-        <v>700</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C72), "ksh", ""))), "")</f>
+        <v>3240</v>
       </c>
       <c r="D71" s="21" t="n">
-        <f aca="false">VALUE(TRIM(raw_data!D71))</f>
-        <v>0.45</v>
+        <f aca="false">VALUE(TRIM(raw_data!D72))</f>
+        <v>0.29</v>
       </c>
       <c r="E71" s="12" t="n">
-        <f aca="false">IF(ISBLANK(raw_data!E71),"",ABS(TRIM(raw_data!E71)))</f>
-        <v>17</v>
+        <f aca="false">IF(ISBLANK(raw_data!E72),"",ABS(TRIM(raw_data!E72)))</f>
+        <v>5</v>
       </c>
       <c r="F71" s="13" t="n">
-        <f aca="false">=IF(ISBLANK(raw_data!F71),"",VALUE(LEFT(raw_data!F71,FIND(" ", raw_data!F71,1))))</f>
-        <v>2.6</v>
+        <f aca="false">=IF(ISBLANK(raw_data!F72),"",VALUE(LEFT(raw_data!F72,FIND(" ", raw_data!F72,1))))</f>
+        <v>3</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="8" t="str">
         <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v>Large Lazy Inflatable Sofa Chairs Pvc Lounger Seat Bag</v>
+        <v>Watercolour Gold Foil Textured Print Pillow Cover</v>
       </c>
       <c r="B72" s="9" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B72), "ksh", ""))), "")</f>
-        <v>2300</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B73), "ksh", ""))), "")</f>
+        <v>345</v>
       </c>
       <c r="C72" s="10" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C72), "ksh", ""))), "")</f>
-        <v>3240</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C73), "ksh", ""))), "")</f>
+        <v>602</v>
       </c>
       <c r="D72" s="21" t="n">
-        <f aca="false">VALUE(TRIM(raw_data!D72))</f>
-        <v>0.29</v>
+        <f aca="false">VALUE(TRIM(raw_data!D73))</f>
+        <v>0.43</v>
       </c>
       <c r="E72" s="12" t="n">
-        <f aca="false">IF(ISBLANK(raw_data!E72),"",ABS(TRIM(raw_data!E72)))</f>
-        <v>5</v>
+        <f aca="false">IF(ISBLANK(raw_data!E73),"",ABS(TRIM(raw_data!E73)))</f>
+        <v>6</v>
       </c>
       <c r="F72" s="13" t="n">
-        <f aca="false">=IF(ISBLANK(raw_data!F72),"",VALUE(LEFT(raw_data!F72,FIND(" ", raw_data!F72,1))))</f>
-        <v>3</v>
+        <f aca="false">=IF(ISBLANK(raw_data!F73),"",VALUE(LEFT(raw_data!F73,FIND(" ", raw_data!F73,1))))</f>
+        <v>2.3</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="8" t="str">
         <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v>Watercolour Gold Foil Textured Print Pillow Cover</v>
+        <v>Wrought Iron Bathroom Shelf Wall Mounted Free Punch Toilet Rack</v>
       </c>
       <c r="B73" s="9" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B73), "ksh", ""))), "")</f>
-        <v>345</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B74), "ksh", ""))), "")</f>
+        <v>509</v>
       </c>
       <c r="C73" s="10" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C73), "ksh", ""))), "")</f>
-        <v>602</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C74), "ksh", ""))), "")</f>
+        <v>899</v>
       </c>
       <c r="D73" s="21" t="n">
-        <f aca="false">VALUE(TRIM(raw_data!D73))</f>
+        <f aca="false">VALUE(TRIM(raw_data!D74))</f>
         <v>0.43</v>
       </c>
       <c r="E73" s="12" t="n">
-        <f aca="false">IF(ISBLANK(raw_data!E73),"",ABS(TRIM(raw_data!E73)))</f>
-        <v>6</v>
+        <f aca="false">IF(ISBLANK(raw_data!E74),"",ABS(TRIM(raw_data!E74)))</f>
+        <v>5</v>
       </c>
       <c r="F73" s="13" t="n">
-        <f aca="false">=IF(ISBLANK(raw_data!F73),"",VALUE(LEFT(raw_data!F73,FIND(" ", raw_data!F73,1))))</f>
-        <v>2.3</v>
+        <f aca="false">=IF(ISBLANK(raw_data!F74),"",VALUE(LEFT(raw_data!F74,FIND(" ", raw_data!F74,1))))</f>
+        <v>3</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="8" t="str">
         <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v>Wrought Iron Bathroom Shelf Wall Mounted Free Punch Toilet Rack</v>
+        <v>7-Piece Set Of Storage Bags, Travel Storage Bags, Shoe Bags</v>
       </c>
       <c r="B74" s="9" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B74), "ksh", ""))), "")</f>
-        <v>509</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B75), "ksh", ""))), "")</f>
+        <v>968</v>
       </c>
       <c r="C74" s="10" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C74), "ksh", ""))), "")</f>
-        <v>899</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C75), "ksh", ""))), "")</f>
+        <v>1814</v>
       </c>
       <c r="D74" s="21" t="n">
-        <f aca="false">VALUE(TRIM(raw_data!D74))</f>
-        <v>0.43</v>
+        <f aca="false">VALUE(TRIM(raw_data!D75))</f>
+        <v>0.47</v>
       </c>
       <c r="E74" s="12" t="n">
-        <f aca="false">IF(ISBLANK(raw_data!E74),"",ABS(TRIM(raw_data!E74)))</f>
-        <v>5</v>
+        <f aca="false">IF(ISBLANK(raw_data!E75),"",ABS(TRIM(raw_data!E75)))</f>
+        <v>6</v>
       </c>
       <c r="F74" s="13" t="n">
-        <f aca="false">=IF(ISBLANK(raw_data!F74),"",VALUE(LEFT(raw_data!F74,FIND(" ", raw_data!F74,1))))</f>
-        <v>3</v>
+        <f aca="false">=IF(ISBLANK(raw_data!F75),"",VALUE(LEFT(raw_data!F75,FIND(" ", raw_data!F75,1))))</f>
+        <v>2.2</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="8" t="str">
         <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v>7-Piece Set Of Storage Bags, Travel Storage Bags, Shoe Bags</v>
+        <v>Electric Led Uv Mosquito Killer Lamp, Outdoor/Indoor Fly Killer Trap Light -Usb</v>
       </c>
       <c r="B75" s="9" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B75), "ksh", ""))), "")</f>
-        <v>968</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B76), "ksh", ""))), "")</f>
+        <v>1570</v>
       </c>
       <c r="C75" s="10" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C75), "ksh", ""))), "")</f>
-        <v>1814</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C76), "ksh", ""))), "")</f>
+        <v>2988</v>
       </c>
       <c r="D75" s="21" t="n">
-        <f aca="false">VALUE(TRIM(raw_data!D75))</f>
+        <f aca="false">VALUE(TRIM(raw_data!D76))</f>
         <v>0.47</v>
       </c>
       <c r="E75" s="12" t="n">
-        <f aca="false">IF(ISBLANK(raw_data!E75),"",ABS(TRIM(raw_data!E75)))</f>
-        <v>6</v>
+        <f aca="false">IF(ISBLANK(raw_data!E76),"",ABS(TRIM(raw_data!E76)))</f>
+        <v>7</v>
       </c>
       <c r="F75" s="13" t="n">
-        <f aca="false">=IF(ISBLANK(raw_data!F75),"",VALUE(LEFT(raw_data!F75,FIND(" ", raw_data!F75,1))))</f>
-        <v>2.2</v>
+        <f aca="false">=IF(ISBLANK(raw_data!F76),"",VALUE(LEFT(raw_data!F76,FIND(" ", raw_data!F76,1))))</f>
+        <v>2.1</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="8" t="str">
         <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v>Electric Led Uv Mosquito Killer Lamp, Outdoor/Indoor Fly Killer Trap Light -Usb</v>
+        <v>2Pcs/Lot Solar Led Outdoor Intelligent Light Controlled Wall Lamp</v>
       </c>
       <c r="B76" s="9" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B76), "ksh", ""))), "")</f>
-        <v>1570</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B77), "ksh", ""))), "")</f>
+        <v>790</v>
       </c>
       <c r="C76" s="10" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C76), "ksh", ""))), "")</f>
-        <v>2988</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C77), "ksh", ""))), "")</f>
+        <v>1485</v>
       </c>
       <c r="D76" s="21" t="n">
-        <f aca="false">VALUE(TRIM(raw_data!D76))</f>
+        <f aca="false">VALUE(TRIM(raw_data!D77))</f>
         <v>0.47</v>
       </c>
-      <c r="E76" s="12" t="n">
-        <f aca="false">IF(ISBLANK(raw_data!E76),"",ABS(TRIM(raw_data!E76)))</f>
-        <v>7</v>
-      </c>
-      <c r="F76" s="13" t="n">
-        <f aca="false">=IF(ISBLANK(raw_data!F76),"",VALUE(LEFT(raw_data!F76,FIND(" ", raw_data!F76,1))))</f>
-        <v>2.1</v>
+      <c r="E76" s="12" t="str">
+        <f aca="false">IF(ISBLANK(raw_data!E77),"",ABS(TRIM(raw_data!E77)))</f>
+        <v/>
+      </c>
+      <c r="F76" s="13" t="str">
+        <f aca="false">=IF(ISBLANK(raw_data!F77),"",VALUE(LEFT(raw_data!F77,FIND(" ", raw_data!F77,1))))</f>
+        <v/>
       </c>
     </row>
     <row r="77" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="8" t="str">
         <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v>2Pcs/Lot Solar Led Outdoor Intelligent Light Controlled Wall Lamp</v>
+        <v>3Pcs Rotary Scraper Thermomix For Kitchen</v>
       </c>
       <c r="B77" s="9" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B77), "ksh", ""))), "")</f>
-        <v>790</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B78), "ksh", ""))), "")</f>
+        <v>690</v>
       </c>
       <c r="C77" s="10" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C77), "ksh", ""))), "")</f>
-        <v>1485</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C78), "ksh", ""))), "")</f>
+        <v>1200</v>
       </c>
       <c r="D77" s="21" t="n">
-        <f aca="false">VALUE(TRIM(raw_data!D77))</f>
-        <v>0.47</v>
+        <f aca="false">VALUE(TRIM(raw_data!D78))</f>
+        <v>0.43</v>
       </c>
       <c r="E77" s="12" t="str">
-        <f aca="false">IF(ISBLANK(raw_data!E77),"",ABS(TRIM(raw_data!E77)))</f>
+        <f aca="false">IF(ISBLANK(raw_data!E78),"",ABS(TRIM(raw_data!E78)))</f>
         <v/>
       </c>
       <c r="F77" s="13" t="str">
-        <f aca="false">=IF(ISBLANK(raw_data!F77),"",VALUE(LEFT(raw_data!F77,FIND(" ", raw_data!F77,1))))</f>
+        <f aca="false">=IF(ISBLANK(raw_data!F78),"",VALUE(LEFT(raw_data!F78,FIND(" ", raw_data!F78,1))))</f>
         <v/>
       </c>
     </row>
     <row r="78" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="8" t="str">
         <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v>3Pcs Rotary Scraper Thermomix For Kitchen</v>
+        <v>Cushion Silicone Butt Cushion Summer Ice Cushion Honeycomb Gel Cushion</v>
       </c>
       <c r="B78" s="9" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B78), "ksh", ""))), "")</f>
-        <v>690</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B79), "ksh", ""))), "")</f>
+        <v>1732</v>
       </c>
       <c r="C78" s="10" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C78), "ksh", ""))), "")</f>
-        <v>1200</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C79), "ksh", ""))), "")</f>
+        <v>1799</v>
       </c>
       <c r="D78" s="21" t="n">
-        <f aca="false">VALUE(TRIM(raw_data!D78))</f>
-        <v>0.43</v>
+        <f aca="false">VALUE(TRIM(raw_data!D79))</f>
+        <v>0.04</v>
       </c>
       <c r="E78" s="12" t="str">
-        <f aca="false">IF(ISBLANK(raw_data!E78),"",ABS(TRIM(raw_data!E78)))</f>
+        <f aca="false">IF(ISBLANK(raw_data!E79),"",ABS(TRIM(raw_data!E79)))</f>
         <v/>
       </c>
       <c r="F78" s="13" t="str">
-        <f aca="false">=IF(ISBLANK(raw_data!F78),"",VALUE(LEFT(raw_data!F78,FIND(" ", raw_data!F78,1))))</f>
+        <f aca="false">=IF(ISBLANK(raw_data!F79),"",VALUE(LEFT(raw_data!F79,FIND(" ", raw_data!F79,1))))</f>
         <v/>
       </c>
     </row>
     <row r="79" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="8" t="str">
         <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v>Cushion Silicone Butt Cushion Summer Ice Cushion Honeycomb Gel Cushion</v>
+        <v>7Pcs Silicone Thumb Knife Finger Protector Vegetable Harvesting Knife</v>
       </c>
       <c r="B79" s="9" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B79), "ksh", ""))), "")</f>
-        <v>1732</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B80), "ksh", ""))), "")</f>
+        <v>230</v>
       </c>
       <c r="C79" s="10" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C79), "ksh", ""))), "")</f>
-        <v>1799</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C80), "ksh", ""))), "")</f>
+        <v>450</v>
       </c>
       <c r="D79" s="21" t="n">
-        <f aca="false">VALUE(TRIM(raw_data!D79))</f>
-        <v>0.04</v>
+        <f aca="false">VALUE(TRIM(raw_data!D80))</f>
+        <v>0.49</v>
       </c>
       <c r="E79" s="12" t="str">
-        <f aca="false">IF(ISBLANK(raw_data!E79),"",ABS(TRIM(raw_data!E79)))</f>
+        <f aca="false">IF(ISBLANK(raw_data!E80),"",ABS(TRIM(raw_data!E80)))</f>
         <v/>
       </c>
       <c r="F79" s="13" t="str">
-        <f aca="false">=IF(ISBLANK(raw_data!F79),"",VALUE(LEFT(raw_data!F79,FIND(" ", raw_data!F79,1))))</f>
+        <f aca="false">=IF(ISBLANK(raw_data!F80),"",VALUE(LEFT(raw_data!F80,FIND(" ", raw_data!F80,1))))</f>
         <v/>
       </c>
     </row>
     <row r="80" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="8" t="str">
         <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v>7Pcs Silicone Thumb Knife Finger Protector Vegetable Harvesting Knife</v>
+        <v>Memory Foam Neck Pillow Cover, With Pillow Core - 50*30Cm</v>
       </c>
       <c r="B80" s="9" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B80), "ksh", ""))), "")</f>
-        <v>230</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B81), "ksh", ""))), "")</f>
+        <v>1189</v>
       </c>
       <c r="C80" s="10" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C80), "ksh", ""))), "")</f>
-        <v>450</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C81), "ksh", ""))), "")</f>
+        <v>2199</v>
       </c>
       <c r="D80" s="21" t="n">
-        <f aca="false">VALUE(TRIM(raw_data!D80))</f>
-        <v>0.49</v>
-      </c>
-      <c r="E80" s="12" t="str">
-        <f aca="false">IF(ISBLANK(raw_data!E80),"",ABS(TRIM(raw_data!E80)))</f>
-        <v/>
-      </c>
-      <c r="F80" s="13" t="str">
-        <f aca="false">=IF(ISBLANK(raw_data!F80),"",VALUE(LEFT(raw_data!F80,FIND(" ", raw_data!F80,1))))</f>
-        <v/>
+        <f aca="false">VALUE(TRIM(raw_data!D81))</f>
+        <v>0.46</v>
+      </c>
+      <c r="E80" s="12" t="n">
+        <f aca="false">IF(ISBLANK(raw_data!E81),"",ABS(TRIM(raw_data!E81)))</f>
+        <v>1</v>
+      </c>
+      <c r="F80" s="13" t="n">
+        <f aca="false">=IF(ISBLANK(raw_data!F81),"",VALUE(LEFT(raw_data!F81,FIND(" ", raw_data!F81,1))))</f>
+        <v>3</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="8" t="str">
         <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v>Memory Foam Neck Pillow Cover, With Pillow Core - 50*30Cm</v>
+        <v>Bedroom Simple Floor Hanging Clothes Rack Single Pole Hat Rack - White</v>
       </c>
       <c r="B81" s="9" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B81), "ksh", ""))), "")</f>
-        <v>1189</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B82), "ksh", ""))), "")</f>
+        <v>979</v>
       </c>
       <c r="C81" s="10" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C81), "ksh", ""))), "")</f>
-        <v>2199</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C82), "ksh", ""))), "")</f>
+        <v>1920</v>
       </c>
       <c r="D81" s="21" t="n">
-        <f aca="false">VALUE(TRIM(raw_data!D81))</f>
-        <v>0.46</v>
+        <f aca="false">VALUE(TRIM(raw_data!D82))</f>
+        <v>0.49</v>
       </c>
       <c r="E81" s="12" t="n">
-        <f aca="false">IF(ISBLANK(raw_data!E81),"",ABS(TRIM(raw_data!E81)))</f>
+        <f aca="false">IF(ISBLANK(raw_data!E82),"",ABS(TRIM(raw_data!E82)))</f>
         <v>1</v>
       </c>
       <c r="F81" s="13" t="n">
-        <f aca="false">=IF(ISBLANK(raw_data!F81),"",VALUE(LEFT(raw_data!F81,FIND(" ", raw_data!F81,1))))</f>
-        <v>3</v>
+        <f aca="false">=IF(ISBLANK(raw_data!F82),"",VALUE(LEFT(raw_data!F82,FIND(" ", raw_data!F82,1))))</f>
+        <v>5</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="8" t="str">
         <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v>Bedroom Simple Floor Hanging Clothes Rack Single Pole Hat Rack - White</v>
+        <v>5M Waterproof Spherical Led String Lights Outdoor Ball Chain Lights Party Lighting Decoration Adjustable</v>
       </c>
       <c r="B82" s="9" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B82), "ksh", ""))), "")</f>
-        <v>979</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B83), "ksh", ""))), "")</f>
+        <v>1460</v>
       </c>
       <c r="C82" s="10" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C82), "ksh", ""))), "")</f>
-        <v>1920</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C83), "ksh", ""))), "")</f>
+        <v>2290</v>
       </c>
       <c r="D82" s="21" t="n">
-        <f aca="false">VALUE(TRIM(raw_data!D82))</f>
-        <v>0.49</v>
-      </c>
-      <c r="E82" s="12" t="n">
-        <f aca="false">IF(ISBLANK(raw_data!E82),"",ABS(TRIM(raw_data!E82)))</f>
-        <v>1</v>
-      </c>
-      <c r="F82" s="13" t="n">
-        <f aca="false">=IF(ISBLANK(raw_data!F82),"",VALUE(LEFT(raw_data!F82,FIND(" ", raw_data!F82,1))))</f>
-        <v>5</v>
+        <f aca="false">VALUE(TRIM(raw_data!D83))</f>
+        <v>0.36</v>
+      </c>
+      <c r="E82" s="12" t="str">
+        <f aca="false">IF(ISBLANK(raw_data!E83),"",ABS(TRIM(raw_data!E83)))</f>
+        <v/>
+      </c>
+      <c r="F82" s="13" t="str">
+        <f aca="false">=IF(ISBLANK(raw_data!F83),"",VALUE(LEFT(raw_data!F83,FIND(" ", raw_data!F83,1))))</f>
+        <v/>
       </c>
     </row>
     <row r="83" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="8" t="str">
         <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v>5M Waterproof Spherical Led String Lights Outdoor Ball Chain Lights Party Lighting Decoration Adjustable</v>
+        <v>2 Pairs Cowhide Split Leather Work Gloves.32Â Or Above Welding Gloves</v>
       </c>
       <c r="B83" s="9" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B83), "ksh", ""))), "")</f>
-        <v>1460</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B84), "ksh", ""))), "")</f>
+        <v>1666</v>
       </c>
       <c r="C83" s="10" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C83), "ksh", ""))), "")</f>
-        <v>2290</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C84), "ksh", ""))), "")</f>
+        <v>1699</v>
       </c>
       <c r="D83" s="21" t="n">
-        <f aca="false">VALUE(TRIM(raw_data!D83))</f>
-        <v>0.36</v>
+        <f aca="false">VALUE(TRIM(raw_data!D84))</f>
+        <v>0.02</v>
       </c>
       <c r="E83" s="12" t="str">
-        <f aca="false">IF(ISBLANK(raw_data!E83),"",ABS(TRIM(raw_data!E83)))</f>
+        <f aca="false">IF(ISBLANK(raw_data!E84),"",ABS(TRIM(raw_data!E84)))</f>
         <v/>
       </c>
       <c r="F83" s="13" t="str">
-        <f aca="false">=IF(ISBLANK(raw_data!F83),"",VALUE(LEFT(raw_data!F83,FIND(" ", raw_data!F83,1))))</f>
+        <f aca="false">=IF(ISBLANK(raw_data!F84),"",VALUE(LEFT(raw_data!F84,FIND(" ", raw_data!F84,1))))</f>
         <v/>
       </c>
     </row>
     <row r="84" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="8" t="str">
         <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v>2 Pairs Cowhide Split Leather Work Gloves.32Â Or Above Welding Gloves</v>
+        <v>Household Pineapple Peeler Peeler</v>
       </c>
       <c r="B84" s="9" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B84), "ksh", ""))), "")</f>
-        <v>1666</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B85), "ksh", ""))), "")</f>
+        <v>330</v>
       </c>
       <c r="C84" s="10" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C84), "ksh", ""))), "")</f>
-        <v>1699</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C85), "ksh", ""))), "")</f>
+        <v>647</v>
       </c>
       <c r="D84" s="21" t="n">
-        <f aca="false">VALUE(TRIM(raw_data!D84))</f>
-        <v>0.02</v>
-      </c>
-      <c r="E84" s="12" t="str">
-        <f aca="false">IF(ISBLANK(raw_data!E84),"",ABS(TRIM(raw_data!E84)))</f>
-        <v/>
-      </c>
-      <c r="F84" s="13" t="str">
-        <f aca="false">=IF(ISBLANK(raw_data!F84),"",VALUE(LEFT(raw_data!F84,FIND(" ", raw_data!F84,1))))</f>
-        <v/>
+        <f aca="false">VALUE(TRIM(raw_data!D85))</f>
+        <v>0.49</v>
+      </c>
+      <c r="E84" s="12" t="n">
+        <f aca="false">IF(ISBLANK(raw_data!E85),"",ABS(TRIM(raw_data!E85)))</f>
+        <v>1</v>
+      </c>
+      <c r="F84" s="13" t="n">
+        <f aca="false">=IF(ISBLANK(raw_data!F85),"",VALUE(LEFT(raw_data!F85,FIND(" ", raw_data!F85,1))))</f>
+        <v>4</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="8" t="str">
         <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v>Household Pineapple Peeler Peeler</v>
+        <v>Creative Owl Shape Keychain Black</v>
       </c>
       <c r="B85" s="9" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B85), "ksh", ""))), "")</f>
-        <v>330</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B87), "ksh", ""))), "")</f>
+        <v>176</v>
       </c>
       <c r="C85" s="10" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C85), "ksh", ""))), "")</f>
-        <v>647</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C87), "ksh", ""))), "")</f>
+        <v>345</v>
       </c>
       <c r="D85" s="21" t="n">
-        <f aca="false">VALUE(TRIM(raw_data!D85))</f>
+        <f aca="false">VALUE(TRIM(raw_data!D87))</f>
         <v>0.49</v>
       </c>
-      <c r="E85" s="12" t="n">
-        <f aca="false">IF(ISBLANK(raw_data!E85),"",ABS(TRIM(raw_data!E85)))</f>
-        <v>1</v>
-      </c>
-      <c r="F85" s="13" t="n">
-        <f aca="false">=IF(ISBLANK(raw_data!F85),"",VALUE(LEFT(raw_data!F85,FIND(" ", raw_data!F85,1))))</f>
-        <v>4</v>
+      <c r="E85" s="12" t="str">
+        <f aca="false">IF(ISBLANK(raw_data!E87),"",ABS(TRIM(raw_data!E87)))</f>
+        <v/>
+      </c>
+      <c r="F85" s="13" t="str">
+        <f aca="false">=IF(ISBLANK(raw_data!F87),"",VALUE(LEFT(raw_data!F87,FIND(" ", raw_data!F87,1))))</f>
+        <v/>
       </c>
     </row>
     <row r="86" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="8" t="str">
         <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v>Balloon Insert, Birthday Party Balloon Set, Pu Leather</v>
+        <v>Office Chair Lumbar Back Support Spine Posture Correction Pillow Car Cushion</v>
       </c>
       <c r="B86" s="9" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B86), "ksh", ""))), "")</f>
-        <v>610</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B88), "ksh", ""))), "")</f>
+        <v>1466</v>
       </c>
       <c r="C86" s="10" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C86), "ksh", ""))), "")</f>
-        <v>1060</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C88), "ksh", ""))), "")</f>
+        <v>1699</v>
       </c>
       <c r="D86" s="21" t="n">
-        <f aca="false">VALUE(TRIM(raw_data!D86))</f>
-        <v>0.42</v>
+        <f aca="false">VALUE(TRIM(raw_data!D88))</f>
+        <v>0.14</v>
       </c>
       <c r="E86" s="12" t="str">
-        <f aca="false">IF(ISBLANK(raw_data!E86),"",ABS(TRIM(raw_data!E86)))</f>
+        <f aca="false">IF(ISBLANK(raw_data!E88),"",ABS(TRIM(raw_data!E88)))</f>
         <v/>
       </c>
       <c r="F86" s="13" t="str">
-        <f aca="false">=IF(ISBLANK(raw_data!F86),"",VALUE(LEFT(raw_data!F86,FIND(" ", raw_data!F86,1))))</f>
+        <f aca="false">=IF(ISBLANK(raw_data!F88),"",VALUE(LEFT(raw_data!F88,FIND(" ", raw_data!F88,1))))</f>
         <v/>
       </c>
     </row>
     <row r="87" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="8" t="str">
         <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v>Creative Owl Shape Keychain Black</v>
+        <v>Cartoon Car Decoration Cute Individuality For Car Home Desk</v>
       </c>
       <c r="B87" s="9" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B87), "ksh", ""))), "")</f>
-        <v>176</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B89), "ksh", ""))), "")</f>
+        <v>274</v>
       </c>
       <c r="C87" s="10" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C87), "ksh", ""))), "")</f>
-        <v>345</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C89), "ksh", ""))), "")</f>
+        <v>537</v>
       </c>
       <c r="D87" s="21" t="n">
-        <f aca="false">VALUE(TRIM(raw_data!D87))</f>
+        <f aca="false">VALUE(TRIM(raw_data!D89))</f>
         <v>0.49</v>
       </c>
       <c r="E87" s="12" t="str">
-        <f aca="false">IF(ISBLANK(raw_data!E87),"",ABS(TRIM(raw_data!E87)))</f>
+        <f aca="false">IF(ISBLANK(raw_data!E89),"",ABS(TRIM(raw_data!E89)))</f>
         <v/>
       </c>
       <c r="F87" s="13" t="str">
-        <f aca="false">=IF(ISBLANK(raw_data!F87),"",VALUE(LEFT(raw_data!F87,FIND(" ", raw_data!F87,1))))</f>
+        <f aca="false">=IF(ISBLANK(raw_data!F89),"",VALUE(LEFT(raw_data!F89,FIND(" ", raw_data!F89,1))))</f>
         <v/>
       </c>
     </row>
     <row r="88" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="8" t="str">
         <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v>Office Chair Lumbar Back Support Spine Posture Correction Pillow Car Cushion</v>
+        <v>Outdoor Portable Water Bottle With Medicine Box - 600Ml - Black</v>
       </c>
       <c r="B88" s="9" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B88), "ksh", ""))), "")</f>
-        <v>1466</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B90), "ksh", ""))), "")</f>
+        <v>799</v>
       </c>
       <c r="C88" s="10" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C88), "ksh", ""))), "")</f>
-        <v>1699</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C90), "ksh", ""))), "")</f>
+        <v>900</v>
       </c>
       <c r="D88" s="21" t="n">
-        <f aca="false">VALUE(TRIM(raw_data!D88))</f>
-        <v>0.14</v>
+        <f aca="false">VALUE(TRIM(raw_data!D90))</f>
+        <v>0.11</v>
       </c>
       <c r="E88" s="12" t="str">
-        <f aca="false">IF(ISBLANK(raw_data!E88),"",ABS(TRIM(raw_data!E88)))</f>
+        <f aca="false">IF(ISBLANK(raw_data!E90),"",ABS(TRIM(raw_data!E90)))</f>
         <v/>
       </c>
       <c r="F88" s="13" t="str">
-        <f aca="false">=IF(ISBLANK(raw_data!F88),"",VALUE(LEFT(raw_data!F88,FIND(" ", raw_data!F88,1))))</f>
+        <f aca="false">=IF(ISBLANK(raw_data!F90),"",VALUE(LEFT(raw_data!F90,FIND(" ", raw_data!F90,1))))</f>
         <v/>
       </c>
     </row>
     <row r="89" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="8" t="str">
         <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v>Cartoon Car Decoration Cute Individuality For Car Home Desk</v>
+        <v>Angle Measuring Tool Full Metal Multi Angle Measuring Tool</v>
       </c>
       <c r="B89" s="9" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B89), "ksh", ""))), "")</f>
-        <v>274</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B91), "ksh", ""))), "")</f>
+        <v>657</v>
       </c>
       <c r="C89" s="10" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C89), "ksh", ""))), "")</f>
-        <v>537</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C91), "ksh", ""))), "")</f>
+        <v>1288</v>
       </c>
       <c r="D89" s="21" t="n">
-        <f aca="false">VALUE(TRIM(raw_data!D89))</f>
+        <f aca="false">VALUE(TRIM(raw_data!D91))</f>
         <v>0.49</v>
       </c>
       <c r="E89" s="12" t="str">
-        <f aca="false">IF(ISBLANK(raw_data!E89),"",ABS(TRIM(raw_data!E89)))</f>
+        <f aca="false">IF(ISBLANK(raw_data!E91),"",ABS(TRIM(raw_data!E91)))</f>
         <v/>
       </c>
       <c r="F89" s="13" t="str">
-        <f aca="false">=IF(ISBLANK(raw_data!F89),"",VALUE(LEFT(raw_data!F89,FIND(" ", raw_data!F89,1))))</f>
+        <f aca="false">=IF(ISBLANK(raw_data!F91),"",VALUE(LEFT(raw_data!F91,FIND(" ", raw_data!F91,1))))</f>
         <v/>
       </c>
     </row>
     <row r="90" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="8" t="str">
         <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v>Outdoor Portable Water Bottle With Medicine Box - 600Ml - Black</v>
+        <v>Wall-Mounted Toothbrush Toothpaste Holder With Multiple Slots</v>
       </c>
       <c r="B90" s="9" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B90), "ksh", ""))), "")</f>
-        <v>799</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B92), "ksh", ""))), "")</f>
+        <v>1468</v>
       </c>
       <c r="C90" s="10" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C90), "ksh", ""))), "")</f>
-        <v>900</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C92), "ksh", ""))), "")</f>
+        <v>1699</v>
       </c>
       <c r="D90" s="21" t="n">
-        <f aca="false">VALUE(TRIM(raw_data!D90))</f>
-        <v>0.11</v>
+        <f aca="false">VALUE(TRIM(raw_data!D92))</f>
+        <v>0.14</v>
       </c>
       <c r="E90" s="12" t="str">
-        <f aca="false">IF(ISBLANK(raw_data!E90),"",ABS(TRIM(raw_data!E90)))</f>
+        <f aca="false">IF(ISBLANK(raw_data!E92),"",ABS(TRIM(raw_data!E92)))</f>
         <v/>
       </c>
       <c r="F90" s="13" t="str">
-        <f aca="false">=IF(ISBLANK(raw_data!F90),"",VALUE(LEFT(raw_data!F90,FIND(" ", raw_data!F90,1))))</f>
+        <f aca="false">=IF(ISBLANK(raw_data!F92),"",VALUE(LEFT(raw_data!F92,FIND(" ", raw_data!F92,1))))</f>
         <v/>
       </c>
     </row>
     <row r="91" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="8" t="str">
         <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v>Angle Measuring Tool Full Metal Multi Angle Measuring Tool</v>
+        <v>Multifunctional Hanging Storage Box Storage Bag (4 Layers)</v>
       </c>
       <c r="B91" s="9" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B91), "ksh", ""))), "")</f>
-        <v>657</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B93), "ksh", ""))), "")</f>
+        <v>630</v>
       </c>
       <c r="C91" s="10" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C91), "ksh", ""))), "")</f>
-        <v>1288</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C93), "ksh", ""))), "")</f>
+        <v>1100</v>
       </c>
       <c r="D91" s="21" t="n">
-        <f aca="false">VALUE(TRIM(raw_data!D91))</f>
-        <v>0.49</v>
+        <f aca="false">VALUE(TRIM(raw_data!D93))</f>
+        <v>0.43</v>
       </c>
       <c r="E91" s="12" t="str">
-        <f aca="false">IF(ISBLANK(raw_data!E91),"",ABS(TRIM(raw_data!E91)))</f>
+        <f aca="false">IF(ISBLANK(raw_data!E93),"",ABS(TRIM(raw_data!E93)))</f>
         <v/>
       </c>
       <c r="F91" s="13" t="str">
-        <f aca="false">=IF(ISBLANK(raw_data!F91),"",VALUE(LEFT(raw_data!F91,FIND(" ", raw_data!F91,1))))</f>
+        <f aca="false">=IF(ISBLANK(raw_data!F93),"",VALUE(LEFT(raw_data!F93,FIND(" ", raw_data!F93,1))))</f>
         <v/>
       </c>
     </row>
     <row r="92" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="8" t="str">
         <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v>Wall-Mounted Toothbrush Toothpaste Holder With Multiple Slots</v>
+        <v>Wall Clock With Hidden Safe Box</v>
       </c>
       <c r="B92" s="9" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B92), "ksh", ""))), "")</f>
-        <v>1468</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B94), "ksh", ""))), "")</f>
+        <v>850</v>
       </c>
       <c r="C92" s="10" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C92), "ksh", ""))), "")</f>
-        <v>1699</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C94), "ksh", ""))), "")</f>
+        <v>1700</v>
       </c>
       <c r="D92" s="21" t="n">
-        <f aca="false">VALUE(TRIM(raw_data!D92))</f>
-        <v>0.14</v>
+        <f aca="false">VALUE(TRIM(raw_data!D94))</f>
+        <v>0.5</v>
       </c>
       <c r="E92" s="12" t="str">
-        <f aca="false">IF(ISBLANK(raw_data!E92),"",ABS(TRIM(raw_data!E92)))</f>
+        <f aca="false">IF(ISBLANK(raw_data!E94),"",ABS(TRIM(raw_data!E94)))</f>
         <v/>
       </c>
       <c r="F92" s="13" t="str">
-        <f aca="false">=IF(ISBLANK(raw_data!F92),"",VALUE(LEFT(raw_data!F92,FIND(" ", raw_data!F92,1))))</f>
+        <f aca="false">=IF(ISBLANK(raw_data!F94),"",VALUE(LEFT(raw_data!F94,FIND(" ", raw_data!F94,1))))</f>
         <v/>
       </c>
     </row>
     <row r="93" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="8" t="str">
         <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v>Multifunctional Hanging Storage Box Storage Bag (4 Layers)</v>
+        <v>Portable Wine Table With Folding Round Table</v>
       </c>
       <c r="B93" s="9" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B93), "ksh", ""))), "")</f>
-        <v>630</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B95), "ksh", ""))), "")</f>
+        <v>1300</v>
       </c>
       <c r="C93" s="10" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C93), "ksh", ""))), "")</f>
-        <v>1100</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C95), "ksh", ""))), "")</f>
+        <v>2500</v>
       </c>
       <c r="D93" s="21" t="n">
-        <f aca="false">VALUE(TRIM(raw_data!D93))</f>
-        <v>0.43</v>
+        <f aca="false">VALUE(TRIM(raw_data!D95))</f>
+        <v>0.48</v>
       </c>
       <c r="E93" s="12" t="str">
-        <f aca="false">IF(ISBLANK(raw_data!E93),"",ABS(TRIM(raw_data!E93)))</f>
+        <f aca="false">IF(ISBLANK(raw_data!E95),"",ABS(TRIM(raw_data!E95)))</f>
         <v/>
       </c>
       <c r="F93" s="13" t="str">
-        <f aca="false">=IF(ISBLANK(raw_data!F93),"",VALUE(LEFT(raw_data!F93,FIND(" ", raw_data!F93,1))))</f>
+        <f aca="false">=IF(ISBLANK(raw_data!F95),"",VALUE(LEFT(raw_data!F95,FIND(" ", raw_data!F95,1))))</f>
         <v/>
       </c>
     </row>
     <row r="94" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="8" t="str">
         <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v>Wall Clock With Hidden Safe Box</v>
+        <v>Sewing Machine Needle Threader Stitch Insertion Tool Automatic Quick Sewing</v>
       </c>
       <c r="B94" s="9" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B94), "ksh", ""))), "")</f>
-        <v>850</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B96), "ksh", ""))), "")</f>
+        <v>105</v>
       </c>
       <c r="C94" s="10" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C94), "ksh", ""))), "")</f>
-        <v>1700</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C96), "ksh", ""))), "")</f>
+        <v>200</v>
       </c>
       <c r="D94" s="21" t="n">
-        <f aca="false">VALUE(TRIM(raw_data!D94))</f>
-        <v>0.5</v>
+        <f aca="false">VALUE(TRIM(raw_data!D96))</f>
+        <v>0.48</v>
       </c>
       <c r="E94" s="12" t="str">
-        <f aca="false">IF(ISBLANK(raw_data!E94),"",ABS(TRIM(raw_data!E94)))</f>
+        <f aca="false">IF(ISBLANK(raw_data!E96),"",ABS(TRIM(raw_data!E96)))</f>
         <v/>
       </c>
       <c r="F94" s="13" t="str">
-        <f aca="false">=IF(ISBLANK(raw_data!F94),"",VALUE(LEFT(raw_data!F94,FIND(" ", raw_data!F94,1))))</f>
+        <f aca="false">=IF(ISBLANK(raw_data!F96),"",VALUE(LEFT(raw_data!F96,FIND(" ", raw_data!F96,1))))</f>
         <v/>
       </c>
     </row>
     <row r="95" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="8" t="str">
         <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v>Portable Wine Table With Folding Round Table</v>
+        <v>6 Layers Steel Pipe Assembling Dustproof Storage Shoe Cabinet</v>
       </c>
       <c r="B95" s="9" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B95), "ksh", ""))), "")</f>
-        <v>1300</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B97), "ksh", ""))), "")</f>
+        <v>899</v>
       </c>
       <c r="C95" s="10" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C95), "ksh", ""))), "")</f>
-        <v>2500</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C97), "ksh", ""))), "")</f>
+        <v>1699</v>
       </c>
       <c r="D95" s="21" t="n">
-        <f aca="false">VALUE(TRIM(raw_data!D95))</f>
-        <v>0.48</v>
+        <f aca="false">VALUE(TRIM(raw_data!D97))</f>
+        <v>0.47</v>
       </c>
       <c r="E95" s="12" t="str">
-        <f aca="false">IF(ISBLANK(raw_data!E95),"",ABS(TRIM(raw_data!E95)))</f>
+        <f aca="false">IF(ISBLANK(raw_data!E97),"",ABS(TRIM(raw_data!E97)))</f>
         <v/>
       </c>
       <c r="F95" s="13" t="str">
-        <f aca="false">=IF(ISBLANK(raw_data!F95),"",VALUE(LEFT(raw_data!F95,FIND(" ", raw_data!F95,1))))</f>
+        <f aca="false">=IF(ISBLANK(raw_data!F97),"",VALUE(LEFT(raw_data!F97,FIND(" ", raw_data!F97,1))))</f>
         <v/>
       </c>
     </row>
     <row r="96" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="8" t="str">
         <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v>Sewing Machine Needle Threader Stitch Insertion Tool Automatic Quick Sewing</v>
+        <v>2Pcs Ice Silk Square Cushion Cover Pillowcases - 65X65Cm</v>
       </c>
       <c r="B96" s="9" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B96), "ksh", ""))), "")</f>
-        <v>105</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B99), "ksh", ""))), "")</f>
+        <v>1200</v>
       </c>
       <c r="C96" s="10" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C96), "ksh", ""))), "")</f>
-        <v>200</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C99), "ksh", ""))), "")</f>
+        <v>2400</v>
       </c>
       <c r="D96" s="21" t="n">
-        <f aca="false">VALUE(TRIM(raw_data!D96))</f>
-        <v>0.48</v>
+        <f aca="false">VALUE(TRIM(raw_data!D99))</f>
+        <v>0.5</v>
       </c>
       <c r="E96" s="12" t="str">
-        <f aca="false">IF(ISBLANK(raw_data!E96),"",ABS(TRIM(raw_data!E96)))</f>
+        <f aca="false">IF(ISBLANK(raw_data!E99),"",ABS(TRIM(raw_data!E99)))</f>
         <v/>
       </c>
       <c r="F96" s="13" t="str">
-        <f aca="false">=IF(ISBLANK(raw_data!F96),"",VALUE(LEFT(raw_data!F96,FIND(" ", raw_data!F96,1))))</f>
+        <f aca="false">=IF(ISBLANK(raw_data!F99),"",VALUE(LEFT(raw_data!F99,FIND(" ", raw_data!F99,1))))</f>
         <v/>
       </c>
     </row>
     <row r="97" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="8" t="str">
         <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v>6 Layers Steel Pipe Assembling Dustproof Storage Shoe Cabinet</v>
+        <v>Wall Mount Automatic Toothpaste Dispenser Toothbrush Holder Toothpaste Squeezer</v>
       </c>
       <c r="B97" s="9" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B97), "ksh", ""))), "")</f>
-        <v>899</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B100), "ksh", ""))), "")</f>
+        <v>1526</v>
       </c>
       <c r="C97" s="10" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C97), "ksh", ""))), "")</f>
-        <v>1699</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C100), "ksh", ""))), "")</f>
+        <v>1660</v>
       </c>
       <c r="D97" s="21" t="n">
-        <f aca="false">VALUE(TRIM(raw_data!D97))</f>
-        <v>0.47</v>
+        <f aca="false">VALUE(TRIM(raw_data!D100))</f>
+        <v>0.08</v>
       </c>
       <c r="E97" s="12" t="str">
-        <f aca="false">IF(ISBLANK(raw_data!E97),"",ABS(TRIM(raw_data!E97)))</f>
+        <f aca="false">IF(ISBLANK(raw_data!E100),"",ABS(TRIM(raw_data!E100)))</f>
         <v/>
       </c>
       <c r="F97" s="13" t="str">
-        <f aca="false">=IF(ISBLANK(raw_data!F97),"",VALUE(LEFT(raw_data!F97,FIND(" ", raw_data!F97,1))))</f>
+        <f aca="false">=IF(ISBLANK(raw_data!F100),"",VALUE(LEFT(raw_data!F100,FIND(" ", raw_data!F100,1))))</f>
         <v/>
       </c>
     </row>
     <row r="98" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="8" t="str">
         <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v>6 Layers Steel Pipe Assembling Dustproof Storage Shoe Cabinet</v>
+        <v>Portable Soap Dispenser Kitchen Detergent Press Box Kitchen Tools</v>
       </c>
       <c r="B98" s="9" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B98), "ksh", ""))), "")</f>
-        <v>899</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B101), "ksh", ""))), "")</f>
+        <v>1462</v>
       </c>
       <c r="C98" s="10" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C98), "ksh", ""))), "")</f>
-        <v>1699</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C101), "ksh", ""))), "")</f>
+        <v>1499</v>
       </c>
       <c r="D98" s="21" t="n">
-        <f aca="false">VALUE(TRIM(raw_data!D98))</f>
-        <v>0.47</v>
+        <f aca="false">VALUE(TRIM(raw_data!D101))</f>
+        <v>0.02</v>
       </c>
       <c r="E98" s="12" t="str">
-        <f aca="false">IF(ISBLANK(raw_data!E98),"",ABS(TRIM(raw_data!E98)))</f>
+        <f aca="false">IF(ISBLANK(raw_data!E101),"",ABS(TRIM(raw_data!E101)))</f>
         <v/>
       </c>
       <c r="F98" s="13" t="str">
-        <f aca="false">=IF(ISBLANK(raw_data!F98),"",VALUE(LEFT(raw_data!F98,FIND(" ", raw_data!F98,1))))</f>
+        <f aca="false">=IF(ISBLANK(raw_data!F101),"",VALUE(LEFT(raw_data!F101,FIND(" ", raw_data!F101,1))))</f>
         <v/>
       </c>
     </row>
     <row r="99" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="8" t="str">
         <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v>2Pcs Ice Silk Square Cushion Cover Pillowcases - 65X65Cm</v>
+        <v>4 Piece Coloured Stainless Steel Kitchenware Set</v>
       </c>
       <c r="B99" s="9" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B99), "ksh", ""))), "")</f>
-        <v>1200</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B102), "ksh", ""))), "")</f>
+        <v>248</v>
       </c>
       <c r="C99" s="10" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C99), "ksh", ""))), "")</f>
-        <v>2400</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C102), "ksh", ""))), "")</f>
+        <v>486</v>
       </c>
       <c r="D99" s="21" t="n">
-        <f aca="false">VALUE(TRIM(raw_data!D99))</f>
-        <v>0.5</v>
+        <f aca="false">VALUE(TRIM(raw_data!D102))</f>
+        <v>0.49</v>
       </c>
       <c r="E99" s="12" t="str">
-        <f aca="false">IF(ISBLANK(raw_data!E99),"",ABS(TRIM(raw_data!E99)))</f>
+        <f aca="false">IF(ISBLANK(raw_data!E102),"",ABS(TRIM(raw_data!E102)))</f>
         <v/>
       </c>
       <c r="F99" s="13" t="str">
-        <f aca="false">=IF(ISBLANK(raw_data!F99),"",VALUE(LEFT(raw_data!F99,FIND(" ", raw_data!F99,1))))</f>
+        <f aca="false">=IF(ISBLANK(raw_data!F102),"",VALUE(LEFT(raw_data!F102,FIND(" ", raw_data!F102,1))))</f>
         <v/>
       </c>
     </row>
     <row r="100" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="8" t="str">
         <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v>Wall Mount Automatic Toothpaste Dispenser Toothbrush Holder Toothpaste Squeezer</v>
+        <v>Metal Wall Clock Silver Dial Crystal Jewelry Round Home Decoration Wall Clock</v>
       </c>
       <c r="B100" s="9" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B100), "ksh", ""))), "")</f>
-        <v>1526</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B103), "ksh", ""))), "")</f>
+        <v>3546</v>
       </c>
       <c r="C100" s="10" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C100), "ksh", ""))), "")</f>
-        <v>1660</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C103), "ksh", ""))), "")</f>
+        <v>3699</v>
       </c>
       <c r="D100" s="21" t="n">
-        <f aca="false">VALUE(TRIM(raw_data!D100))</f>
-        <v>0.08</v>
+        <f aca="false">VALUE(TRIM(raw_data!D103))</f>
+        <v>0.04</v>
       </c>
       <c r="E100" s="12" t="str">
-        <f aca="false">IF(ISBLANK(raw_data!E100),"",ABS(TRIM(raw_data!E100)))</f>
+        <f aca="false">IF(ISBLANK(raw_data!E103),"",ABS(TRIM(raw_data!E103)))</f>
         <v/>
       </c>
       <c r="F100" s="13" t="str">
-        <f aca="false">=IF(ISBLANK(raw_data!F100),"",VALUE(LEFT(raw_data!F100,FIND(" ", raw_data!F100,1))))</f>
+        <f aca="false">=IF(ISBLANK(raw_data!F103),"",VALUE(LEFT(raw_data!F103,FIND(" ", raw_data!F103,1))))</f>
         <v/>
       </c>
     </row>
     <row r="101" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="8" t="str">
         <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v>Portable Soap Dispenser Kitchen Detergent Press Box Kitchen Tools</v>
+        <v>Baby Early Education Shape And Color Cognitive Training Toys</v>
       </c>
       <c r="B101" s="9" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B101), "ksh", ""))), "")</f>
-        <v>1462</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B104), "ksh", ""))), "")</f>
+        <v>525</v>
       </c>
       <c r="C101" s="10" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C101), "ksh", ""))), "")</f>
-        <v>1499</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C104), "ksh", ""))), "")</f>
+        <v>1029</v>
       </c>
       <c r="D101" s="21" t="n">
-        <f aca="false">VALUE(TRIM(raw_data!D101))</f>
-        <v>0.02</v>
+        <f aca="false">VALUE(TRIM(raw_data!D104))</f>
+        <v>0.49</v>
       </c>
       <c r="E101" s="12" t="str">
-        <f aca="false">IF(ISBLANK(raw_data!E101),"",ABS(TRIM(raw_data!E101)))</f>
+        <f aca="false">IF(ISBLANK(raw_data!E104),"",ABS(TRIM(raw_data!E104)))</f>
         <v/>
       </c>
       <c r="F101" s="13" t="str">
-        <f aca="false">=IF(ISBLANK(raw_data!F101),"",VALUE(LEFT(raw_data!F101,FIND(" ", raw_data!F101,1))))</f>
+        <f aca="false">=IF(ISBLANK(raw_data!F104),"",VALUE(LEFT(raw_data!F104,FIND(" ", raw_data!F104,1))))</f>
         <v/>
       </c>
     </row>
     <row r="102" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="8" t="str">
         <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v>4 Piece Coloured Stainless Steel Kitchenware Set</v>
+        <v>8In1 Screwdriver With Led Light</v>
       </c>
       <c r="B102" s="9" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B102), "ksh", ""))), "")</f>
-        <v>248</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B105), "ksh", ""))), "")</f>
+        <v>1080</v>
       </c>
       <c r="C102" s="10" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C102), "ksh", ""))), "")</f>
-        <v>486</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C105), "ksh", ""))), "")</f>
+        <v>1874</v>
       </c>
       <c r="D102" s="21" t="n">
-        <f aca="false">VALUE(TRIM(raw_data!D102))</f>
-        <v>0.49</v>
+        <f aca="false">VALUE(TRIM(raw_data!D105))</f>
+        <v>0.42</v>
       </c>
       <c r="E102" s="12" t="str">
-        <f aca="false">IF(ISBLANK(raw_data!E102),"",ABS(TRIM(raw_data!E102)))</f>
+        <f aca="false">IF(ISBLANK(raw_data!E105),"",ABS(TRIM(raw_data!E105)))</f>
         <v/>
       </c>
       <c r="F102" s="13" t="str">
-        <f aca="false">=IF(ISBLANK(raw_data!F102),"",VALUE(LEFT(raw_data!F102,FIND(" ", raw_data!F102,1))))</f>
+        <f aca="false">=IF(ISBLANK(raw_data!F105),"",VALUE(LEFT(raw_data!F105,FIND(" ", raw_data!F105,1))))</f>
         <v/>
       </c>
     </row>
     <row r="103" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="8" t="str">
         <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v>Metal Wall Clock Silver Dial Crystal Jewelry Round Home Decoration Wall Clock</v>
+        <v>Konka Healty Electric Kettle, 24-Hour Heat Preservation,1.5L,800W, White</v>
       </c>
       <c r="B103" s="9" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B103), "ksh", ""))), "")</f>
-        <v>3546</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B106), "ksh", ""))), "")</f>
+        <v>3640</v>
       </c>
       <c r="C103" s="10" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C103), "ksh", ""))), "")</f>
-        <v>3699</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C106), "ksh", ""))), "")</f>
+        <v>4588</v>
       </c>
       <c r="D103" s="21" t="n">
-        <f aca="false">VALUE(TRIM(raw_data!D103))</f>
-        <v>0.04</v>
-      </c>
-      <c r="E103" s="12" t="str">
-        <f aca="false">IF(ISBLANK(raw_data!E103),"",ABS(TRIM(raw_data!E103)))</f>
-        <v/>
-      </c>
-      <c r="F103" s="13" t="str">
-        <f aca="false">=IF(ISBLANK(raw_data!F103),"",VALUE(LEFT(raw_data!F103,FIND(" ", raw_data!F103,1))))</f>
-        <v/>
+        <f aca="false">VALUE(TRIM(raw_data!D106))</f>
+        <v>0.21</v>
+      </c>
+      <c r="E103" s="12" t="n">
+        <f aca="false">IF(ISBLANK(raw_data!E106),"",ABS(TRIM(raw_data!E106)))</f>
+        <v>1</v>
+      </c>
+      <c r="F103" s="13" t="n">
+        <f aca="false">=IF(ISBLANK(raw_data!F106),"",VALUE(LEFT(raw_data!F106,FIND(" ", raw_data!F106,1))))</f>
+        <v>5</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="8" t="str">
         <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v>Baby Early Education Shape And Color Cognitive Training Toys</v>
+        <v>9Pcs Gas Mask, For Painting, Dust, Formaldehyde Grinding, Polishing</v>
       </c>
       <c r="B104" s="9" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B104), "ksh", ""))), "")</f>
-        <v>525</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B107), "ksh", ""))), "")</f>
+        <v>1420</v>
       </c>
       <c r="C104" s="10" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C104), "ksh", ""))), "")</f>
-        <v>1029</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C107), "ksh", ""))), "")</f>
+        <v>2420</v>
       </c>
       <c r="D104" s="21" t="n">
-        <f aca="false">VALUE(TRIM(raw_data!D104))</f>
-        <v>0.49</v>
+        <f aca="false">VALUE(TRIM(raw_data!D107))</f>
+        <v>0.41</v>
       </c>
       <c r="E104" s="12" t="str">
-        <f aca="false">IF(ISBLANK(raw_data!E104),"",ABS(TRIM(raw_data!E104)))</f>
+        <f aca="false">IF(ISBLANK(raw_data!E107),"",ABS(TRIM(raw_data!E107)))</f>
         <v/>
       </c>
       <c r="F104" s="13" t="str">
-        <f aca="false">=IF(ISBLANK(raw_data!F104),"",VALUE(LEFT(raw_data!F104,FIND(" ", raw_data!F104,1))))</f>
+        <f aca="false">=IF(ISBLANK(raw_data!F107),"",VALUE(LEFT(raw_data!F107,FIND(" ", raw_data!F107,1))))</f>
         <v/>
       </c>
     </row>
     <row r="105" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="8" t="str">
         <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v>8In1 Screwdriver With Led Light</v>
+        <v>24 Grid Wall-Mounted Sundries Organiser Fabric Closet Bag Storage Rack</v>
       </c>
       <c r="B105" s="9" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B105), "ksh", ""))), "")</f>
-        <v>1080</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B108), "ksh", ""))), "")</f>
+        <v>1875</v>
       </c>
       <c r="C105" s="10" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C105), "ksh", ""))), "")</f>
-        <v>1874</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C108), "ksh", ""))), "")</f>
+        <v>1899</v>
       </c>
       <c r="D105" s="21" t="n">
-        <f aca="false">VALUE(TRIM(raw_data!D105))</f>
-        <v>0.42</v>
+        <f aca="false">VALUE(TRIM(raw_data!D108))</f>
+        <v>0.01</v>
       </c>
       <c r="E105" s="12" t="str">
-        <f aca="false">IF(ISBLANK(raw_data!E105),"",ABS(TRIM(raw_data!E105)))</f>
+        <f aca="false">IF(ISBLANK(raw_data!E108),"",ABS(TRIM(raw_data!E108)))</f>
         <v/>
       </c>
       <c r="F105" s="13" t="str">
-        <f aca="false">=IF(ISBLANK(raw_data!F105),"",VALUE(LEFT(raw_data!F105,FIND(" ", raw_data!F105,1))))</f>
+        <f aca="false">=IF(ISBLANK(raw_data!F108),"",VALUE(LEFT(raw_data!F108,FIND(" ", raw_data!F108,1))))</f>
         <v/>
       </c>
     </row>
     <row r="106" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="8" t="str">
         <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v>Konka Healty Electric Kettle, 24-Hour Heat Preservation,1.5L,800W, White</v>
+        <v>1Pc Refrigerator Food Seal Pocket Fridge Bags</v>
       </c>
       <c r="B106" s="9" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B106), "ksh", ""))), "")</f>
-        <v>3640</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B109), "ksh", ""))), "")</f>
+        <v>198</v>
       </c>
       <c r="C106" s="10" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C106), "ksh", ""))), "")</f>
-        <v>4588</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C109), "ksh", ""))), "")</f>
+        <v>260</v>
       </c>
       <c r="D106" s="21" t="n">
-        <f aca="false">VALUE(TRIM(raw_data!D106))</f>
-        <v>0.21</v>
-      </c>
-      <c r="E106" s="12" t="n">
-        <f aca="false">IF(ISBLANK(raw_data!E106),"",ABS(TRIM(raw_data!E106)))</f>
-        <v>1</v>
-      </c>
-      <c r="F106" s="13" t="n">
-        <f aca="false">=IF(ISBLANK(raw_data!F106),"",VALUE(LEFT(raw_data!F106,FIND(" ", raw_data!F106,1))))</f>
-        <v>5</v>
+        <f aca="false">VALUE(TRIM(raw_data!D109))</f>
+        <v>0.24</v>
+      </c>
+      <c r="E106" s="12" t="str">
+        <f aca="false">IF(ISBLANK(raw_data!E109),"",ABS(TRIM(raw_data!E109)))</f>
+        <v/>
+      </c>
+      <c r="F106" s="13" t="str">
+        <f aca="false">=IF(ISBLANK(raw_data!F109),"",VALUE(LEFT(raw_data!F109,FIND(" ", raw_data!F109,1))))</f>
+        <v/>
       </c>
     </row>
     <row r="107" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="8" t="str">
         <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v>9Pcs Gas Mask, For Painting, Dust, Formaldehyde Grinding, Polishing</v>
+        <v>Led Solar Street Light-Fake Camera</v>
       </c>
       <c r="B107" s="9" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B107), "ksh", ""))), "")</f>
-        <v>1420</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B110), "ksh", ""))), "")</f>
+        <v>1150</v>
       </c>
       <c r="C107" s="10" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C107), "ksh", ""))), "")</f>
-        <v>2420</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C110), "ksh", ""))), "")</f>
+        <v>1737</v>
       </c>
       <c r="D107" s="21" t="n">
-        <f aca="false">VALUE(TRIM(raw_data!D107))</f>
-        <v>0.41</v>
+        <f aca="false">VALUE(TRIM(raw_data!D110))</f>
+        <v>0.34</v>
       </c>
       <c r="E107" s="12" t="str">
-        <f aca="false">IF(ISBLANK(raw_data!E107),"",ABS(TRIM(raw_data!E107)))</f>
+        <f aca="false">IF(ISBLANK(raw_data!E110),"",ABS(TRIM(raw_data!E110)))</f>
         <v/>
       </c>
       <c r="F107" s="13" t="str">
-        <f aca="false">=IF(ISBLANK(raw_data!F107),"",VALUE(LEFT(raw_data!F107,FIND(" ", raw_data!F107,1))))</f>
+        <f aca="false">=IF(ISBLANK(raw_data!F110),"",VALUE(LEFT(raw_data!F110,FIND(" ", raw_data!F110,1))))</f>
         <v/>
       </c>
     </row>
     <row r="108" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="8" t="str">
         <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v>24 Grid Wall-Mounted Sundries Organiser Fabric Closet Bag Storage Rack</v>
+        <v>Cartoon Embroidered Mini Towel Bear Cotton Wash Cloth Hand 4Pcs</v>
       </c>
       <c r="B108" s="9" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B108), "ksh", ""))), "")</f>
-        <v>1875</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B111), "ksh", ""))), "")</f>
+        <v>1190</v>
       </c>
       <c r="C108" s="10" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C108), "ksh", ""))), "")</f>
-        <v>1899</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C111), "ksh", ""))), "")</f>
+        <v>1810</v>
       </c>
       <c r="D108" s="21" t="n">
-        <f aca="false">VALUE(TRIM(raw_data!D108))</f>
-        <v>0.01</v>
+        <f aca="false">VALUE(TRIM(raw_data!D111))</f>
+        <v>0.34</v>
       </c>
       <c r="E108" s="12" t="str">
-        <f aca="false">IF(ISBLANK(raw_data!E108),"",ABS(TRIM(raw_data!E108)))</f>
+        <f aca="false">IF(ISBLANK(raw_data!E111),"",ABS(TRIM(raw_data!E111)))</f>
         <v/>
       </c>
       <c r="F108" s="13" t="str">
-        <f aca="false">=IF(ISBLANK(raw_data!F108),"",VALUE(LEFT(raw_data!F108,FIND(" ", raw_data!F108,1))))</f>
+        <f aca="false">=IF(ISBLANK(raw_data!F111),"",VALUE(LEFT(raw_data!F111,FIND(" ", raw_data!F111,1))))</f>
         <v/>
       </c>
     </row>
     <row r="109" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="8" t="str">
         <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v>1Pc Refrigerator Food Seal Pocket Fridge Bags</v>
+        <v>Shower Nozzle Cleaning Unclogging Needle Mini Crevice Small Hole Cleaning Brush</v>
       </c>
       <c r="B109" s="9" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B109), "ksh", ""))), "")</f>
-        <v>198</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B112), "ksh", ""))), "")</f>
+        <v>1658</v>
       </c>
       <c r="C109" s="10" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C109), "ksh", ""))), "")</f>
-        <v>260</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C112), "ksh", ""))), "")</f>
+        <v>1699</v>
       </c>
       <c r="D109" s="21" t="n">
-        <f aca="false">VALUE(TRIM(raw_data!D109))</f>
-        <v>0.24</v>
+        <f aca="false">VALUE(TRIM(raw_data!D112))</f>
+        <v>0.02</v>
       </c>
       <c r="E109" s="12" t="str">
-        <f aca="false">IF(ISBLANK(raw_data!E109),"",ABS(TRIM(raw_data!E109)))</f>
+        <f aca="false">IF(ISBLANK(raw_data!E112),"",ABS(TRIM(raw_data!E112)))</f>
         <v/>
       </c>
       <c r="F109" s="13" t="str">
-        <f aca="false">=IF(ISBLANK(raw_data!F109),"",VALUE(LEFT(raw_data!F109,FIND(" ", raw_data!F109,1))))</f>
+        <f aca="false">=IF(ISBLANK(raw_data!F112),"",VALUE(LEFT(raw_data!F112,FIND(" ", raw_data!F112,1))))</f>
         <v/>
       </c>
     </row>
     <row r="110" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="8" t="str">
         <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v>Led Solar Street Light-Fake Camera</v>
+        <v>Thickening Multipurpose Non Stick Easy To Clean Heat Resistant Spoon Pad</v>
       </c>
       <c r="B110" s="9" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B110), "ksh", ""))), "")</f>
-        <v>1150</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B113), "ksh", ""))), "")</f>
+        <v>1768</v>
       </c>
       <c r="C110" s="10" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C110), "ksh", ""))), "")</f>
-        <v>1737</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C113), "ksh", ""))), "")</f>
+        <v>1799</v>
       </c>
       <c r="D110" s="21" t="n">
-        <f aca="false">VALUE(TRIM(raw_data!D110))</f>
-        <v>0.34</v>
+        <f aca="false">VALUE(TRIM(raw_data!D113))</f>
+        <v>0.02</v>
       </c>
       <c r="E110" s="12" t="str">
-        <f aca="false">IF(ISBLANK(raw_data!E110),"",ABS(TRIM(raw_data!E110)))</f>
+        <f aca="false">IF(ISBLANK(raw_data!E113),"",ABS(TRIM(raw_data!E113)))</f>
         <v/>
       </c>
       <c r="F110" s="13" t="str">
-        <f aca="false">=IF(ISBLANK(raw_data!F110),"",VALUE(LEFT(raw_data!F110,FIND(" ", raw_data!F110,1))))</f>
+        <f aca="false">=IF(ISBLANK(raw_data!F113),"",VALUE(LEFT(raw_data!F113,FIND(" ", raw_data!F113,1))))</f>
         <v/>
       </c>
     </row>
     <row r="111" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A111" s="8" t="str">
         <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v>Cartoon Embroidered Mini Towel Bear Cotton Wash Cloth Hand 4Pcs</v>
+        <v>6 In 1 Bottle Can Opener Multifunctional Easy Opener</v>
       </c>
       <c r="B111" s="9" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B111), "ksh", ""))), "")</f>
-        <v>1190</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B114), "ksh", ""))), "")</f>
+        <v>199</v>
       </c>
       <c r="C111" s="10" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C111), "ksh", ""))), "")</f>
-        <v>1810</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C114), "ksh", ""))), "")</f>
+        <v>553</v>
       </c>
       <c r="D111" s="21" t="n">
-        <f aca="false">VALUE(TRIM(raw_data!D111))</f>
-        <v>0.34</v>
+        <f aca="false">VALUE(TRIM(raw_data!D114))</f>
+        <v>0.64</v>
       </c>
       <c r="E111" s="12" t="str">
-        <f aca="false">IF(ISBLANK(raw_data!E111),"",ABS(TRIM(raw_data!E111)))</f>
+        <f aca="false">IF(ISBLANK(raw_data!E114),"",ABS(TRIM(raw_data!E114)))</f>
         <v/>
       </c>
       <c r="F111" s="13" t="str">
-        <f aca="false">=IF(ISBLANK(raw_data!F111),"",VALUE(LEFT(raw_data!F111,FIND(" ", raw_data!F111,1))))</f>
+        <f aca="false">=IF(ISBLANK(raw_data!F114),"",VALUE(LEFT(raw_data!F114,FIND(" ", raw_data!F114,1))))</f>
         <v/>
       </c>
     </row>
     <row r="112" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A112" s="8" t="str">
         <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v>Shower Nozzle Cleaning Unclogging Needle Mini Crevice Small Hole Cleaning Brush</v>
+        <v>Wall-Mounted Sticker Punch-Free Plug Fixer</v>
       </c>
       <c r="B112" s="9" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B112), "ksh", ""))), "")</f>
-        <v>1658</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B115), "ksh", ""))), "")</f>
+        <v>450</v>
       </c>
       <c r="C112" s="10" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C112), "ksh", ""))), "")</f>
-        <v>1699</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C115), "ksh", ""))), "")</f>
+        <v>900</v>
       </c>
       <c r="D112" s="21" t="n">
-        <f aca="false">VALUE(TRIM(raw_data!D112))</f>
-        <v>0.02</v>
-      </c>
-      <c r="E112" s="12" t="str">
-        <f aca="false">IF(ISBLANK(raw_data!E112),"",ABS(TRIM(raw_data!E112)))</f>
-        <v/>
-      </c>
-      <c r="F112" s="13" t="str">
-        <f aca="false">=IF(ISBLANK(raw_data!F112),"",VALUE(LEFT(raw_data!F112,FIND(" ", raw_data!F112,1))))</f>
-        <v/>
+        <f aca="false">VALUE(TRIM(raw_data!D115))</f>
+        <v>0.5</v>
+      </c>
+      <c r="E112" s="12" t="n">
+        <f aca="false">IF(ISBLANK(raw_data!E115),"",ABS(TRIM(raw_data!E115)))</f>
+        <v>1</v>
+      </c>
+      <c r="F112" s="13" t="n">
+        <f aca="false">=IF(ISBLANK(raw_data!F115),"",VALUE(LEFT(raw_data!F115,FIND(" ", raw_data!F115,1))))</f>
+        <v>2</v>
       </c>
     </row>
     <row r="113" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A113" s="8" t="str">
         <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v>Thickening Multipurpose Non Stick Easy To Clean Heat Resistant Spoon Pad</v>
+        <v>Black Simple Water Cup Wine Coaster Anti Slip Absorbent</v>
       </c>
       <c r="B113" s="9" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B113), "ksh", ""))), "")</f>
-        <v>1768</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B116), "ksh", ""))), "")</f>
+        <v>169</v>
       </c>
       <c r="C113" s="10" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C113), "ksh", ""))), "")</f>
-        <v>1799</v>
+        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C116), "ksh", ""))), "")</f>
+        <v>320</v>
       </c>
       <c r="D113" s="21" t="n">
-        <f aca="false">VALUE(TRIM(raw_data!D113))</f>
-        <v>0.02</v>
+        <f aca="false">VALUE(TRIM(raw_data!D116))</f>
+        <v>0.47</v>
       </c>
       <c r="E113" s="12" t="str">
-        <f aca="false">IF(ISBLANK(raw_data!E113),"",ABS(TRIM(raw_data!E113)))</f>
+        <f aca="false">IF(ISBLANK(raw_data!E116),"",ABS(TRIM(raw_data!E116)))</f>
         <v/>
       </c>
       <c r="F113" s="13" t="str">
-        <f aca="false">=IF(ISBLANK(raw_data!F113),"",VALUE(LEFT(raw_data!F113,FIND(" ", raw_data!F113,1))))</f>
+        <f aca="false">=IF(ISBLANK(raw_data!F116),"",VALUE(LEFT(raw_data!F116,FIND(" ", raw_data!F116,1))))</f>
         <v/>
       </c>
     </row>
     <row r="114" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A114" s="8" t="str">
         <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v>6 In 1 Bottle Can Opener Multifunctional Easy Opener</v>
-      </c>
-      <c r="B114" s="9" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B114), "ksh", ""))), "")</f>
-        <v>199</v>
-      </c>
-      <c r="C114" s="10" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C114), "ksh", ""))), "")</f>
-        <v>553</v>
-      </c>
-      <c r="D114" s="21" t="n">
-        <f aca="false">VALUE(TRIM(raw_data!D114))</f>
-        <v>0.64</v>
-      </c>
-      <c r="E114" s="12" t="str">
-        <f aca="false">IF(ISBLANK(raw_data!E114),"",ABS(TRIM(raw_data!E114)))</f>
-        <v/>
-      </c>
-      <c r="F114" s="13" t="str">
-        <f aca="false">=IF(ISBLANK(raw_data!F114),"",VALUE(LEFT(raw_data!F114,FIND(" ", raw_data!F114,1))))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="115" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A115" s="8" t="str">
-        <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v>Wall-Mounted Sticker Punch-Free Plug Fixer</v>
-      </c>
-      <c r="B115" s="9" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B115), "ksh", ""))), "")</f>
-        <v>450</v>
-      </c>
-      <c r="C115" s="10" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C115), "ksh", ""))), "")</f>
-        <v>900</v>
-      </c>
-      <c r="D115" s="21" t="n">
-        <f aca="false">VALUE(TRIM(raw_data!D115))</f>
-        <v>0.5</v>
-      </c>
-      <c r="E115" s="12" t="n">
-        <f aca="false">IF(ISBLANK(raw_data!E115),"",ABS(TRIM(raw_data!E115)))</f>
-        <v>1</v>
-      </c>
-      <c r="F115" s="13" t="n">
-        <f aca="false">=IF(ISBLANK(raw_data!F115),"",VALUE(LEFT(raw_data!F115,FIND(" ", raw_data!F115,1))))</f>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="116" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A116" s="8" t="str">
-        <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v>Black Simple Water Cup Wine Coaster Anti Slip Absorbent</v>
-      </c>
-      <c r="B116" s="9" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!B116), "ksh", ""))), "")</f>
-        <v>169</v>
-      </c>
-      <c r="C116" s="10" t="n">
-        <f aca="false">IFERROR(VALUE(TRIM(SUBSTITUTE(LOWER(raw_data!C116), "ksh", ""))), "")</f>
-        <v>320</v>
-      </c>
-      <c r="D116" s="21" t="n">
-        <f aca="false">VALUE(TRIM(raw_data!D116))</f>
-        <v>0.47</v>
-      </c>
-      <c r="E116" s="12" t="str">
-        <f aca="false">IF(ISBLANK(raw_data!E116),"",ABS(TRIM(raw_data!E116)))</f>
-        <v/>
-      </c>
-      <c r="F116" s="13" t="str">
-        <f aca="false">=IF(ISBLANK(raw_data!F116),"",VALUE(LEFT(raw_data!F116,FIND(" ", raw_data!F116,1))))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="117" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A117" s="8" t="str">
-        <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="118" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A118" s="8" t="str">
-        <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="119" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A119" s="8" t="str">
-        <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="120" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A120" s="8" t="str">
-        <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="121" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A121" s="8" t="str">
-        <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="122" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A122" s="8" t="str">
-        <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="123" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A123" s="8" t="str">
-        <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="124" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A124" s="8" t="str">
-        <f aca="false">PROPER(TRIM(raw_data!A:A))</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F124"/>
+  <autoFilter ref="A1:F114"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>

<commit_message>
Categorise rating handle the uncategorised range
</commit_message>
<xml_diff>
--- a/dashboard/jumia_product_dashboard.xlsx
+++ b/dashboard/jumia_product_dashboard.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="raw_data" sheetId="1" state="visible" r:id="rId3"/>
@@ -13,7 +13,7 @@
     <sheet name="clean_data" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">clean_data!$A$1:$G$114</definedName>
+    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">clean_data!$A$1:$L$114</definedName>
     <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">raw_data!$A:$I</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="700" uniqueCount="419">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="705" uniqueCount="424">
   <si>
     <t xml:space="preserve">Product</t>
   </si>
@@ -1303,6 +1303,15 @@
     <t xml:space="preserve">=COUNTIF($clean_data.G:G, "&lt;&gt;0")</t>
   </si>
   <si>
+    <t xml:space="preserve">rating categories</t>
+  </si>
+  <si>
+    <t xml:space="preserve">range from 4.1 – 4.5 is not categorised</t>
+  </si>
+  <si>
+    <t xml:space="preserve">move ange for average to 4.5 – only use clean_rating_category in analysis</t>
+  </si>
+  <si>
     <t xml:space="preserve">clean_products</t>
   </si>
   <si>
@@ -1333,7 +1342,13 @@
     <t xml:space="preserve">validation_percentage_discount</t>
   </si>
   <si>
-    <t xml:space="preserve">clean_discount_amount</t>
+    <t xml:space="preserve">clean_discounted_amount</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rating_category</t>
+  </si>
+  <si>
+    <t xml:space="preserve">clean_rating_categories</t>
   </si>
 </sst>
 </file>
@@ -1581,7 +1596,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="9">
+  <dxfs count="15">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -1656,6 +1671,30 @@
       </font>
     </dxf>
     <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFFCC"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF996600"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFFFF"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
       <font>
         <name val="Arial"/>
         <charset val="1"/>
@@ -1665,6 +1704,49 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFCCFFCC"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <charset val="1"/>
+        <family val="2"/>
+        <b val="1"/>
+        <color rgb="FFFFFFFF"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFCC0000"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <charset val="1"/>
+        <family val="2"/>
+        <color rgb="FFCC0000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFCCCC"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <charset val="1"/>
+        <family val="2"/>
+        <color rgb="FF996600"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFFCC"/>
         </patternFill>
       </fill>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
@@ -1683,7 +1765,7 @@
       <rgbColor rgb="FF800000"/>
       <rgbColor rgb="FF006600"/>
       <rgbColor rgb="FF000080"/>
-      <rgbColor rgb="FF808000"/>
+      <rgbColor rgb="FF996600"/>
       <rgbColor rgb="FF800080"/>
       <rgbColor rgb="FF008080"/>
       <rgbColor rgb="FFC0C0C0"/>
@@ -4215,14 +4297,14 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B2:F16"/>
+  <dimension ref="B2:F17"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="4" width="11.53"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="4" width="17.39"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="4" width="27.26"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="4" width="23.65"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="4" width="39.55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="4" width="57.36"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="4" width="53.84"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="7" style="4" width="11.53"/>
   </cols>
@@ -4449,6 +4531,20 @@
       </c>
       <c r="F16" s="4" t="s">
         <v>407</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B17" s="4" t="s">
+        <v>408</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>409</v>
+      </c>
+      <c r="D17" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="E17" s="4" t="s">
+        <v>410</v>
       </c>
     </row>
   </sheetData>
@@ -4467,7 +4563,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K116"/>
+  <dimension ref="A1:M116"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="13.2" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="7" width="68.58"/>
@@ -4481,42 +4577,50 @@
     <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="9" min="9" style="7" width="27.26"/>
     <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="10" min="10" style="7" width="33.8"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="7" width="23.79"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="12" style="7" width="11.53"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="12" min="12" style="7" width="22.4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="7" width="30.74"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="14" style="7" width="11.53"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="13" t="s">
-        <v>408</v>
+        <v>411</v>
       </c>
       <c r="B1" s="14" t="s">
-        <v>409</v>
+        <v>412</v>
       </c>
       <c r="C1" s="14" t="s">
-        <v>410</v>
+        <v>413</v>
       </c>
       <c r="D1" s="15" t="s">
-        <v>411</v>
+        <v>414</v>
       </c>
       <c r="E1" s="16" t="s">
-        <v>412</v>
+        <v>415</v>
       </c>
       <c r="F1" s="17" t="s">
-        <v>413</v>
+        <v>416</v>
       </c>
       <c r="G1" s="18" t="s">
-        <v>414</v>
+        <v>417</v>
       </c>
       <c r="H1" s="19" t="s">
-        <v>415</v>
+        <v>418</v>
       </c>
       <c r="I1" s="19" t="s">
-        <v>416</v>
+        <v>419</v>
       </c>
       <c r="J1" s="19" t="s">
-        <v>417</v>
+        <v>420</v>
       </c>
       <c r="K1" s="20" t="s">
-        <v>418</v>
+        <v>421</v>
+      </c>
+      <c r="L1" s="19" t="s">
+        <v>422</v>
+      </c>
+      <c r="M1" s="19" t="s">
+        <v>423</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4564,6 +4668,14 @@
         <f aca="false">IFERROR(C2-B2,"")</f>
         <v/>
       </c>
+      <c r="L2" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F2), "MISSING", IF(F2&lt;3, "POOR", IF(F2&gt;4.5, "EXCELLENT", IF(AND(F2&gt;=3, F2&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>UN-CATEGORISED</v>
+      </c>
+      <c r="M2" s="7" t="str">
+        <f aca="false">IF(L2="UN-CATEGORISED", "AVERAGE", L2)</f>
+        <v>AVERAGE</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="str">
@@ -4610,6 +4722,14 @@
         <f aca="false">IFERROR(C3-B3,"")</f>
         <v>1526</v>
       </c>
+      <c r="L3" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F3), "MISSING", IF(F3&lt;3, "POOR", IF(F3&gt;4.5, "EXCELLENT", IF(AND(F3&gt;=3, F3&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>EXCELLENT</v>
+      </c>
+      <c r="M3" s="7" t="str">
+        <f aca="false">IF(L3="UN-CATEGORISED", "AVERAGE", L3)</f>
+        <v>EXCELLENT</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="str">
@@ -4656,6 +4776,14 @@
         <f aca="false">IFERROR(C4-B4,"")</f>
         <v>42</v>
       </c>
+      <c r="L4" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F4), "MISSING", IF(F4&lt;3, "POOR", IF(F4&gt;4.5, "EXCELLENT", IF(AND(F4&gt;=3, F4&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>AVERAGE</v>
+      </c>
+      <c r="M4" s="7" t="str">
+        <f aca="false">IF(L4="UN-CATEGORISED", "AVERAGE", L4)</f>
+        <v>AVERAGE</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="str">
@@ -4702,6 +4830,14 @@
         <f aca="false">IFERROR(C5-B5,"")</f>
         <v>189</v>
       </c>
+      <c r="L5" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F5), "MISSING", IF(F5&lt;3, "POOR", IF(F5&gt;4.5, "EXCELLENT", IF(AND(F5&gt;=3, F5&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>EXCELLENT</v>
+      </c>
+      <c r="M5" s="7" t="str">
+        <f aca="false">IF(L5="UN-CATEGORISED", "AVERAGE", L5)</f>
+        <v>EXCELLENT</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="str">
@@ -4748,6 +4884,14 @@
         <f aca="false">IFERROR(C6-B6,"")</f>
         <v>510</v>
       </c>
+      <c r="L6" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F6), "MISSING", IF(F6&lt;3, "POOR", IF(F6&gt;4.5, "EXCELLENT", IF(AND(F6&gt;=3, F6&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>EXCELLENT</v>
+      </c>
+      <c r="M6" s="7" t="str">
+        <f aca="false">IF(L6="UN-CATEGORISED", "AVERAGE", L6)</f>
+        <v>EXCELLENT</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="str">
@@ -4794,6 +4938,14 @@
         <f aca="false">IFERROR(C7-B7,"")</f>
         <v>95</v>
       </c>
+      <c r="L7" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F7), "MISSING", IF(F7&lt;3, "POOR", IF(F7&gt;4.5, "EXCELLENT", IF(AND(F7&gt;=3, F7&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>EXCELLENT</v>
+      </c>
+      <c r="M7" s="7" t="str">
+        <f aca="false">IF(L7="UN-CATEGORISED", "AVERAGE", L7)</f>
+        <v>EXCELLENT</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="str">
@@ -4840,6 +4992,14 @@
         <f aca="false">IFERROR(C8-B8,"")</f>
         <v>544</v>
       </c>
+      <c r="L8" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F8), "MISSING", IF(F8&lt;3, "POOR", IF(F8&gt;4.5, "EXCELLENT", IF(AND(F8&gt;=3, F8&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>EXCELLENT</v>
+      </c>
+      <c r="M8" s="7" t="str">
+        <f aca="false">IF(L8="UN-CATEGORISED", "AVERAGE", L8)</f>
+        <v>EXCELLENT</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="str">
@@ -4886,6 +5046,14 @@
         <f aca="false">IFERROR(C9-B9,"")</f>
         <v>713</v>
       </c>
+      <c r="L9" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F9), "MISSING", IF(F9&lt;3, "POOR", IF(F9&gt;4.5, "EXCELLENT", IF(AND(F9&gt;=3, F9&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>EXCELLENT</v>
+      </c>
+      <c r="M9" s="7" t="str">
+        <f aca="false">IF(L9="UN-CATEGORISED", "AVERAGE", L9)</f>
+        <v>EXCELLENT</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="str">
@@ -4932,6 +5100,14 @@
         <f aca="false">IFERROR(C10-B10,"")</f>
         <v>305</v>
       </c>
+      <c r="L10" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F10), "MISSING", IF(F10&lt;3, "POOR", IF(F10&gt;4.5, "EXCELLENT", IF(AND(F10&gt;=3, F10&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>EXCELLENT</v>
+      </c>
+      <c r="M10" s="7" t="str">
+        <f aca="false">IF(L10="UN-CATEGORISED", "AVERAGE", L10)</f>
+        <v>EXCELLENT</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="str">
@@ -4978,6 +5154,14 @@
         <f aca="false">IFERROR(C11-B11,"")</f>
         <v>1011</v>
       </c>
+      <c r="L11" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F11), "MISSING", IF(F11&lt;3, "POOR", IF(F11&gt;4.5, "EXCELLENT", IF(AND(F11&gt;=3, F11&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>EXCELLENT</v>
+      </c>
+      <c r="M11" s="7" t="str">
+        <f aca="false">IF(L11="UN-CATEGORISED", "AVERAGE", L11)</f>
+        <v>EXCELLENT</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="str">
@@ -5024,6 +5208,14 @@
         <f aca="false">IFERROR(C12-B12,"")</f>
         <v>335</v>
       </c>
+      <c r="L12" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F12), "MISSING", IF(F12&lt;3, "POOR", IF(F12&gt;4.5, "EXCELLENT", IF(AND(F12&gt;=3, F12&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>POOR</v>
+      </c>
+      <c r="M12" s="7" t="str">
+        <f aca="false">IF(L12="UN-CATEGORISED", "AVERAGE", L12)</f>
+        <v>POOR</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="str">
@@ -5070,6 +5262,14 @@
         <f aca="false">IFERROR(C13-B13,"")</f>
         <v>528</v>
       </c>
+      <c r="L13" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F13), "MISSING", IF(F13&lt;3, "POOR", IF(F13&gt;4.5, "EXCELLENT", IF(AND(F13&gt;=3, F13&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>AVERAGE</v>
+      </c>
+      <c r="M13" s="7" t="str">
+        <f aca="false">IF(L13="UN-CATEGORISED", "AVERAGE", L13)</f>
+        <v>AVERAGE</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="str">
@@ -5116,6 +5316,14 @@
         <f aca="false">IFERROR(C14-B14,"")</f>
         <v>401</v>
       </c>
+      <c r="L14" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F14), "MISSING", IF(F14&lt;3, "POOR", IF(F14&gt;4.5, "EXCELLENT", IF(AND(F14&gt;=3, F14&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>EXCELLENT</v>
+      </c>
+      <c r="M14" s="7" t="str">
+        <f aca="false">IF(L14="UN-CATEGORISED", "AVERAGE", L14)</f>
+        <v>EXCELLENT</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="str">
@@ -5162,6 +5370,14 @@
         <f aca="false">IFERROR(C15-B15,"")</f>
         <v>197</v>
       </c>
+      <c r="L15" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F15), "MISSING", IF(F15&lt;3, "POOR", IF(F15&gt;4.5, "EXCELLENT", IF(AND(F15&gt;=3, F15&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>UN-CATEGORISED</v>
+      </c>
+      <c r="M15" s="7" t="str">
+        <f aca="false">IF(L15="UN-CATEGORISED", "AVERAGE", L15)</f>
+        <v>AVERAGE</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="str">
@@ -5208,6 +5424,14 @@
         <f aca="false">IFERROR(C16-B16,"")</f>
         <v>231</v>
       </c>
+      <c r="L16" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F16), "MISSING", IF(F16&lt;3, "POOR", IF(F16&gt;4.5, "EXCELLENT", IF(AND(F16&gt;=3, F16&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>EXCELLENT</v>
+      </c>
+      <c r="M16" s="7" t="str">
+        <f aca="false">IF(L16="UN-CATEGORISED", "AVERAGE", L16)</f>
+        <v>EXCELLENT</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="str">
@@ -5254,6 +5478,14 @@
         <f aca="false">IFERROR(C17-B17,"")</f>
         <v>719</v>
       </c>
+      <c r="L17" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F17), "MISSING", IF(F17&lt;3, "POOR", IF(F17&gt;4.5, "EXCELLENT", IF(AND(F17&gt;=3, F17&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>UN-CATEGORISED</v>
+      </c>
+      <c r="M17" s="7" t="str">
+        <f aca="false">IF(L17="UN-CATEGORISED", "AVERAGE", L17)</f>
+        <v>AVERAGE</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="str">
@@ -5300,6 +5532,14 @@
         <f aca="false">IFERROR(C18-B18,"")</f>
         <v>846</v>
       </c>
+      <c r="L18" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F18), "MISSING", IF(F18&lt;3, "POOR", IF(F18&gt;4.5, "EXCELLENT", IF(AND(F18&gt;=3, F18&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>POOR</v>
+      </c>
+      <c r="M18" s="7" t="str">
+        <f aca="false">IF(L18="UN-CATEGORISED", "AVERAGE", L18)</f>
+        <v>POOR</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="str">
@@ -5346,6 +5586,14 @@
         <f aca="false">IFERROR(C19-B19,"")</f>
         <v>741</v>
       </c>
+      <c r="L19" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F19), "MISSING", IF(F19&lt;3, "POOR", IF(F19&gt;4.5, "EXCELLENT", IF(AND(F19&gt;=3, F19&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>UN-CATEGORISED</v>
+      </c>
+      <c r="M19" s="7" t="str">
+        <f aca="false">IF(L19="UN-CATEGORISED", "AVERAGE", L19)</f>
+        <v>AVERAGE</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="str">
@@ -5392,6 +5640,14 @@
         <f aca="false">IFERROR(C20-B20,"")</f>
         <v>948</v>
       </c>
+      <c r="L20" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F20), "MISSING", IF(F20&lt;3, "POOR", IF(F20&gt;4.5, "EXCELLENT", IF(AND(F20&gt;=3, F20&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>EXCELLENT</v>
+      </c>
+      <c r="M20" s="7" t="str">
+        <f aca="false">IF(L20="UN-CATEGORISED", "AVERAGE", L20)</f>
+        <v>EXCELLENT</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="str">
@@ -5438,6 +5694,14 @@
         <f aca="false">IFERROR(C21-B21,"")</f>
         <v>483</v>
       </c>
+      <c r="L21" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F21), "MISSING", IF(F21&lt;3, "POOR", IF(F21&gt;4.5, "EXCELLENT", IF(AND(F21&gt;=3, F21&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>EXCELLENT</v>
+      </c>
+      <c r="M21" s="7" t="str">
+        <f aca="false">IF(L21="UN-CATEGORISED", "AVERAGE", L21)</f>
+        <v>EXCELLENT</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="str">
@@ -5484,6 +5748,14 @@
         <f aca="false">IFERROR(C22-B22,"")</f>
         <v>40</v>
       </c>
+      <c r="L22" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F22), "MISSING", IF(F22&lt;3, "POOR", IF(F22&gt;4.5, "EXCELLENT", IF(AND(F22&gt;=3, F22&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>EXCELLENT</v>
+      </c>
+      <c r="M22" s="7" t="str">
+        <f aca="false">IF(L22="UN-CATEGORISED", "AVERAGE", L22)</f>
+        <v>EXCELLENT</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="str">
@@ -5530,6 +5802,14 @@
         <f aca="false">IFERROR(C23-B23,"")</f>
         <v>257</v>
       </c>
+      <c r="L23" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F23), "MISSING", IF(F23&lt;3, "POOR", IF(F23&gt;4.5, "EXCELLENT", IF(AND(F23&gt;=3, F23&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>POOR</v>
+      </c>
+      <c r="M23" s="7" t="str">
+        <f aca="false">IF(L23="UN-CATEGORISED", "AVERAGE", L23)</f>
+        <v>POOR</v>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="str">
@@ -5576,6 +5856,14 @@
         <f aca="false">IFERROR(C24-B24,"")</f>
         <v>575</v>
       </c>
+      <c r="L24" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F24), "MISSING", IF(F24&lt;3, "POOR", IF(F24&gt;4.5, "EXCELLENT", IF(AND(F24&gt;=3, F24&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>UN-CATEGORISED</v>
+      </c>
+      <c r="M24" s="7" t="str">
+        <f aca="false">IF(L24="UN-CATEGORISED", "AVERAGE", L24)</f>
+        <v>AVERAGE</v>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="7" t="str">
@@ -5622,6 +5910,14 @@
         <f aca="false">IFERROR(C25-B25,"")</f>
         <v>267</v>
       </c>
+      <c r="L25" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F25), "MISSING", IF(F25&lt;3, "POOR", IF(F25&gt;4.5, "EXCELLENT", IF(AND(F25&gt;=3, F25&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>UN-CATEGORISED</v>
+      </c>
+      <c r="M25" s="7" t="str">
+        <f aca="false">IF(L25="UN-CATEGORISED", "AVERAGE", L25)</f>
+        <v>AVERAGE</v>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="7" t="str">
@@ -5668,6 +5964,14 @@
         <f aca="false">IFERROR(C26-B26,"")</f>
         <v>37</v>
       </c>
+      <c r="L26" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F26), "MISSING", IF(F26&lt;3, "POOR", IF(F26&gt;4.5, "EXCELLENT", IF(AND(F26&gt;=3, F26&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>EXCELLENT</v>
+      </c>
+      <c r="M26" s="7" t="str">
+        <f aca="false">IF(L26="UN-CATEGORISED", "AVERAGE", L26)</f>
+        <v>EXCELLENT</v>
+      </c>
     </row>
     <row r="27" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="7" t="str">
@@ -5714,6 +6018,14 @@
         <f aca="false">IFERROR(C27-B27,"")</f>
         <v>233</v>
       </c>
+      <c r="L27" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F27), "MISSING", IF(F27&lt;3, "POOR", IF(F27&gt;4.5, "EXCELLENT", IF(AND(F27&gt;=3, F27&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>EXCELLENT</v>
+      </c>
+      <c r="M27" s="7" t="str">
+        <f aca="false">IF(L27="UN-CATEGORISED", "AVERAGE", L27)</f>
+        <v>EXCELLENT</v>
+      </c>
     </row>
     <row r="28" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="7" t="str">
@@ -5760,6 +6072,14 @@
         <f aca="false">IFERROR(C28-B28,"")</f>
         <v>67</v>
       </c>
+      <c r="L28" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F28), "MISSING", IF(F28&lt;3, "POOR", IF(F28&gt;4.5, "EXCELLENT", IF(AND(F28&gt;=3, F28&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>EXCELLENT</v>
+      </c>
+      <c r="M28" s="7" t="str">
+        <f aca="false">IF(L28="UN-CATEGORISED", "AVERAGE", L28)</f>
+        <v>EXCELLENT</v>
+      </c>
     </row>
     <row r="29" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="7" t="str">
@@ -5806,6 +6126,14 @@
         <f aca="false">IFERROR(C29-B29,"")</f>
         <v>31</v>
       </c>
+      <c r="L29" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F29), "MISSING", IF(F29&lt;3, "POOR", IF(F29&gt;4.5, "EXCELLENT", IF(AND(F29&gt;=3, F29&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>EXCELLENT</v>
+      </c>
+      <c r="M29" s="7" t="str">
+        <f aca="false">IF(L29="UN-CATEGORISED", "AVERAGE", L29)</f>
+        <v>EXCELLENT</v>
+      </c>
     </row>
     <row r="30" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="7" t="str">
@@ -5852,6 +6180,14 @@
         <f aca="false">IFERROR(C30-B30,"")</f>
         <v>470</v>
       </c>
+      <c r="L30" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F30), "MISSING", IF(F30&lt;3, "POOR", IF(F30&gt;4.5, "EXCELLENT", IF(AND(F30&gt;=3, F30&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>EXCELLENT</v>
+      </c>
+      <c r="M30" s="7" t="str">
+        <f aca="false">IF(L30="UN-CATEGORISED", "AVERAGE", L30)</f>
+        <v>EXCELLENT</v>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="7" t="str">
@@ -5898,6 +6234,14 @@
         <f aca="false">IFERROR(C31-B31,"")</f>
         <v>359</v>
       </c>
+      <c r="L31" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F31), "MISSING", IF(F31&lt;3, "POOR", IF(F31&gt;4.5, "EXCELLENT", IF(AND(F31&gt;=3, F31&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>UN-CATEGORISED</v>
+      </c>
+      <c r="M31" s="7" t="str">
+        <f aca="false">IF(L31="UN-CATEGORISED", "AVERAGE", L31)</f>
+        <v>AVERAGE</v>
+      </c>
     </row>
     <row r="32" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="7" t="str">
@@ -5944,6 +6288,14 @@
         <f aca="false">IFERROR(C32-B32,"")</f>
         <v>724</v>
       </c>
+      <c r="L32" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F32), "MISSING", IF(F32&lt;3, "POOR", IF(F32&gt;4.5, "EXCELLENT", IF(AND(F32&gt;=3, F32&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>EXCELLENT</v>
+      </c>
+      <c r="M32" s="7" t="str">
+        <f aca="false">IF(L32="UN-CATEGORISED", "AVERAGE", L32)</f>
+        <v>EXCELLENT</v>
+      </c>
     </row>
     <row r="33" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="7" t="str">
@@ -5990,6 +6342,14 @@
         <f aca="false">IFERROR(C33-B33,"")</f>
         <v>919</v>
       </c>
+      <c r="L33" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F33), "MISSING", IF(F33&lt;3, "POOR", IF(F33&gt;4.5, "EXCELLENT", IF(AND(F33&gt;=3, F33&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>EXCELLENT</v>
+      </c>
+      <c r="M33" s="7" t="str">
+        <f aca="false">IF(L33="UN-CATEGORISED", "AVERAGE", L33)</f>
+        <v>EXCELLENT</v>
+      </c>
     </row>
     <row r="34" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="7" t="str">
@@ -6036,6 +6396,14 @@
         <f aca="false">IFERROR(C34-B34,"")</f>
         <v>819</v>
       </c>
+      <c r="L34" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F34), "MISSING", IF(F34&lt;3, "POOR", IF(F34&gt;4.5, "EXCELLENT", IF(AND(F34&gt;=3, F34&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>UN-CATEGORISED</v>
+      </c>
+      <c r="M34" s="7" t="str">
+        <f aca="false">IF(L34="UN-CATEGORISED", "AVERAGE", L34)</f>
+        <v>AVERAGE</v>
+      </c>
     </row>
     <row r="35" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="7" t="str">
@@ -6082,6 +6450,14 @@
         <f aca="false">IFERROR(C35-B35,"")</f>
         <v>1070</v>
       </c>
+      <c r="L35" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F35), "MISSING", IF(F35&lt;3, "POOR", IF(F35&gt;4.5, "EXCELLENT", IF(AND(F35&gt;=3, F35&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>EXCELLENT</v>
+      </c>
+      <c r="M35" s="7" t="str">
+        <f aca="false">IF(L35="UN-CATEGORISED", "AVERAGE", L35)</f>
+        <v>EXCELLENT</v>
+      </c>
     </row>
     <row r="36" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="7" t="str">
@@ -6128,6 +6504,14 @@
         <f aca="false">IFERROR(C36-B36,"")</f>
         <v>710</v>
       </c>
+      <c r="L36" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F36), "MISSING", IF(F36&lt;3, "POOR", IF(F36&gt;4.5, "EXCELLENT", IF(AND(F36&gt;=3, F36&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>EXCELLENT</v>
+      </c>
+      <c r="M36" s="7" t="str">
+        <f aca="false">IF(L36="UN-CATEGORISED", "AVERAGE", L36)</f>
+        <v>EXCELLENT</v>
+      </c>
     </row>
     <row r="37" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="7" t="str">
@@ -6174,6 +6558,14 @@
         <f aca="false">IFERROR(C37-B37,"")</f>
         <v>587</v>
       </c>
+      <c r="L37" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F37), "MISSING", IF(F37&lt;3, "POOR", IF(F37&gt;4.5, "EXCELLENT", IF(AND(F37&gt;=3, F37&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>EXCELLENT</v>
+      </c>
+      <c r="M37" s="7" t="str">
+        <f aca="false">IF(L37="UN-CATEGORISED", "AVERAGE", L37)</f>
+        <v>EXCELLENT</v>
+      </c>
     </row>
     <row r="38" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="7" t="str">
@@ -6220,6 +6612,14 @@
         <f aca="false">IFERROR(C38-B38,"")</f>
         <v>695</v>
       </c>
+      <c r="L38" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F38), "MISSING", IF(F38&lt;3, "POOR", IF(F38&gt;4.5, "EXCELLENT", IF(AND(F38&gt;=3, F38&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>EXCELLENT</v>
+      </c>
+      <c r="M38" s="7" t="str">
+        <f aca="false">IF(L38="UN-CATEGORISED", "AVERAGE", L38)</f>
+        <v>EXCELLENT</v>
+      </c>
     </row>
     <row r="39" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="7" t="str">
@@ -6266,6 +6666,14 @@
         <f aca="false">IFERROR(C39-B39,"")</f>
         <v>470</v>
       </c>
+      <c r="L39" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F39), "MISSING", IF(F39&lt;3, "POOR", IF(F39&gt;4.5, "EXCELLENT", IF(AND(F39&gt;=3, F39&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>AVERAGE</v>
+      </c>
+      <c r="M39" s="7" t="str">
+        <f aca="false">IF(L39="UN-CATEGORISED", "AVERAGE", L39)</f>
+        <v>AVERAGE</v>
+      </c>
     </row>
     <row r="40" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="7" t="str">
@@ -6312,6 +6720,14 @@
         <f aca="false">IFERROR(C40-B40,"")</f>
         <v>165</v>
       </c>
+      <c r="L40" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F40), "MISSING", IF(F40&lt;3, "POOR", IF(F40&gt;4.5, "EXCELLENT", IF(AND(F40&gt;=3, F40&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>EXCELLENT</v>
+      </c>
+      <c r="M40" s="7" t="str">
+        <f aca="false">IF(L40="UN-CATEGORISED", "AVERAGE", L40)</f>
+        <v>EXCELLENT</v>
+      </c>
     </row>
     <row r="41" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="7" t="str">
@@ -6358,6 +6774,14 @@
         <f aca="false">IFERROR(C41-B41,"")</f>
         <v>291</v>
       </c>
+      <c r="L41" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F41), "MISSING", IF(F41&lt;3, "POOR", IF(F41&gt;4.5, "EXCELLENT", IF(AND(F41&gt;=3, F41&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>AVERAGE</v>
+      </c>
+      <c r="M41" s="7" t="str">
+        <f aca="false">IF(L41="UN-CATEGORISED", "AVERAGE", L41)</f>
+        <v>AVERAGE</v>
+      </c>
     </row>
     <row r="42" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="7" t="str">
@@ -6404,6 +6828,14 @@
         <f aca="false">IFERROR(C42-B42,"")</f>
         <v>1670</v>
       </c>
+      <c r="L42" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F42), "MISSING", IF(F42&lt;3, "POOR", IF(F42&gt;4.5, "EXCELLENT", IF(AND(F42&gt;=3, F42&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>UN-CATEGORISED</v>
+      </c>
+      <c r="M42" s="7" t="str">
+        <f aca="false">IF(L42="UN-CATEGORISED", "AVERAGE", L42)</f>
+        <v>AVERAGE</v>
+      </c>
     </row>
     <row r="43" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="7" t="str">
@@ -6450,6 +6882,14 @@
         <f aca="false">IFERROR(C43-B43,"")</f>
         <v>62</v>
       </c>
+      <c r="L43" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F43), "MISSING", IF(F43&lt;3, "POOR", IF(F43&gt;4.5, "EXCELLENT", IF(AND(F43&gt;=3, F43&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>EXCELLENT</v>
+      </c>
+      <c r="M43" s="7" t="str">
+        <f aca="false">IF(L43="UN-CATEGORISED", "AVERAGE", L43)</f>
+        <v>EXCELLENT</v>
+      </c>
     </row>
     <row r="44" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="7" t="str">
@@ -6496,6 +6936,14 @@
         <f aca="false">IFERROR(C44-B44,"")</f>
         <v>220</v>
       </c>
+      <c r="L44" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F44), "MISSING", IF(F44&lt;3, "POOR", IF(F44&gt;4.5, "EXCELLENT", IF(AND(F44&gt;=3, F44&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>EXCELLENT</v>
+      </c>
+      <c r="M44" s="7" t="str">
+        <f aca="false">IF(L44="UN-CATEGORISED", "AVERAGE", L44)</f>
+        <v>EXCELLENT</v>
+      </c>
     </row>
     <row r="45" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="7" t="str">
@@ -6542,6 +6990,14 @@
         <f aca="false">IFERROR(C45-B45,"")</f>
         <v>700</v>
       </c>
+      <c r="L45" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F45), "MISSING", IF(F45&lt;3, "POOR", IF(F45&gt;4.5, "EXCELLENT", IF(AND(F45&gt;=3, F45&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>EXCELLENT</v>
+      </c>
+      <c r="M45" s="7" t="str">
+        <f aca="false">IF(L45="UN-CATEGORISED", "AVERAGE", L45)</f>
+        <v>EXCELLENT</v>
+      </c>
     </row>
     <row r="46" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="7" t="str">
@@ -6588,6 +7044,14 @@
         <f aca="false">IFERROR(C46-B46,"")</f>
         <v>1010</v>
       </c>
+      <c r="L46" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F46), "MISSING", IF(F46&lt;3, "POOR", IF(F46&gt;4.5, "EXCELLENT", IF(AND(F46&gt;=3, F46&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>AVERAGE</v>
+      </c>
+      <c r="M46" s="7" t="str">
+        <f aca="false">IF(L46="UN-CATEGORISED", "AVERAGE", L46)</f>
+        <v>AVERAGE</v>
+      </c>
     </row>
     <row r="47" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="7" t="str">
@@ -6634,6 +7098,14 @@
         <f aca="false">IFERROR(C47-B47,"")</f>
         <v>33</v>
       </c>
+      <c r="L47" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F47), "MISSING", IF(F47&lt;3, "POOR", IF(F47&gt;4.5, "EXCELLENT", IF(AND(F47&gt;=3, F47&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>EXCELLENT</v>
+      </c>
+      <c r="M47" s="7" t="str">
+        <f aca="false">IF(L47="UN-CATEGORISED", "AVERAGE", L47)</f>
+        <v>EXCELLENT</v>
+      </c>
     </row>
     <row r="48" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="7" t="str">
@@ -6680,6 +7152,14 @@
         <f aca="false">IFERROR(C48-B48,"")</f>
         <v>644</v>
       </c>
+      <c r="L48" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F48), "MISSING", IF(F48&lt;3, "POOR", IF(F48&gt;4.5, "EXCELLENT", IF(AND(F48&gt;=3, F48&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>EXCELLENT</v>
+      </c>
+      <c r="M48" s="7" t="str">
+        <f aca="false">IF(L48="UN-CATEGORISED", "AVERAGE", L48)</f>
+        <v>EXCELLENT</v>
+      </c>
     </row>
     <row r="49" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="7" t="str">
@@ -6726,6 +7206,14 @@
         <f aca="false">IFERROR(C49-B49,"")</f>
         <v>2393</v>
       </c>
+      <c r="L49" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F49), "MISSING", IF(F49&lt;3, "POOR", IF(F49&gt;4.5, "EXCELLENT", IF(AND(F49&gt;=3, F49&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>AVERAGE</v>
+      </c>
+      <c r="M49" s="7" t="str">
+        <f aca="false">IF(L49="UN-CATEGORISED", "AVERAGE", L49)</f>
+        <v>AVERAGE</v>
+      </c>
     </row>
     <row r="50" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="7" t="str">
@@ -6772,6 +7260,14 @@
         <f aca="false">IFERROR(C50-B50,"")</f>
         <v>238</v>
       </c>
+      <c r="L50" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F50), "MISSING", IF(F50&lt;3, "POOR", IF(F50&gt;4.5, "EXCELLENT", IF(AND(F50&gt;=3, F50&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>EXCELLENT</v>
+      </c>
+      <c r="M50" s="7" t="str">
+        <f aca="false">IF(L50="UN-CATEGORISED", "AVERAGE", L50)</f>
+        <v>EXCELLENT</v>
+      </c>
     </row>
     <row r="51" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="7" t="str">
@@ -6818,6 +7314,14 @@
         <f aca="false">IFERROR(C51-B51,"")</f>
         <v>456</v>
       </c>
+      <c r="L51" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F51), "MISSING", IF(F51&lt;3, "POOR", IF(F51&gt;4.5, "EXCELLENT", IF(AND(F51&gt;=3, F51&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>EXCELLENT</v>
+      </c>
+      <c r="M51" s="7" t="str">
+        <f aca="false">IF(L51="UN-CATEGORISED", "AVERAGE", L51)</f>
+        <v>EXCELLENT</v>
+      </c>
     </row>
     <row r="52" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="7" t="str">
@@ -6864,6 +7368,14 @@
         <f aca="false">IFERROR(C52-B52,"")</f>
         <v>263</v>
       </c>
+      <c r="L52" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F52), "MISSING", IF(F52&lt;3, "POOR", IF(F52&gt;4.5, "EXCELLENT", IF(AND(F52&gt;=3, F52&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>EXCELLENT</v>
+      </c>
+      <c r="M52" s="7" t="str">
+        <f aca="false">IF(L52="UN-CATEGORISED", "AVERAGE", L52)</f>
+        <v>EXCELLENT</v>
+      </c>
     </row>
     <row r="53" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="7" t="str">
@@ -6910,6 +7422,14 @@
         <f aca="false">IFERROR(C53-B53,"")</f>
         <v>504</v>
       </c>
+      <c r="L53" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F53), "MISSING", IF(F53&lt;3, "POOR", IF(F53&gt;4.5, "EXCELLENT", IF(AND(F53&gt;=3, F53&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>EXCELLENT</v>
+      </c>
+      <c r="M53" s="7" t="str">
+        <f aca="false">IF(L53="UN-CATEGORISED", "AVERAGE", L53)</f>
+        <v>EXCELLENT</v>
+      </c>
     </row>
     <row r="54" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="7" t="str">
@@ -6956,6 +7476,14 @@
         <f aca="false">IFERROR(C54-B54,"")</f>
         <v>169</v>
       </c>
+      <c r="L54" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F54), "MISSING", IF(F54&lt;3, "POOR", IF(F54&gt;4.5, "EXCELLENT", IF(AND(F54&gt;=3, F54&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>EXCELLENT</v>
+      </c>
+      <c r="M54" s="7" t="str">
+        <f aca="false">IF(L54="UN-CATEGORISED", "AVERAGE", L54)</f>
+        <v>EXCELLENT</v>
+      </c>
     </row>
     <row r="55" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="7" t="str">
@@ -7002,6 +7530,14 @@
         <f aca="false">IFERROR(C55-B55,"")</f>
         <v>631</v>
       </c>
+      <c r="L55" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F55), "MISSING", IF(F55&lt;3, "POOR", IF(F55&gt;4.5, "EXCELLENT", IF(AND(F55&gt;=3, F55&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>EXCELLENT</v>
+      </c>
+      <c r="M55" s="7" t="str">
+        <f aca="false">IF(L55="UN-CATEGORISED", "AVERAGE", L55)</f>
+        <v>EXCELLENT</v>
+      </c>
     </row>
     <row r="56" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="7" t="str">
@@ -7048,6 +7584,14 @@
         <f aca="false">IFERROR(C56-B56,"")</f>
         <v>510</v>
       </c>
+      <c r="L56" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F56), "MISSING", IF(F56&lt;3, "POOR", IF(F56&gt;4.5, "EXCELLENT", IF(AND(F56&gt;=3, F56&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>EXCELLENT</v>
+      </c>
+      <c r="M56" s="7" t="str">
+        <f aca="false">IF(L56="UN-CATEGORISED", "AVERAGE", L56)</f>
+        <v>EXCELLENT</v>
+      </c>
     </row>
     <row r="57" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="7" t="str">
@@ -7094,6 +7638,14 @@
         <f aca="false">IFERROR(C57-B57,"")</f>
         <v>238</v>
       </c>
+      <c r="L57" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F57), "MISSING", IF(F57&lt;3, "POOR", IF(F57&gt;4.5, "EXCELLENT", IF(AND(F57&gt;=3, F57&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>EXCELLENT</v>
+      </c>
+      <c r="M57" s="7" t="str">
+        <f aca="false">IF(L57="UN-CATEGORISED", "AVERAGE", L57)</f>
+        <v>EXCELLENT</v>
+      </c>
     </row>
     <row r="58" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="7" t="str">
@@ -7140,6 +7692,14 @@
         <f aca="false">IFERROR(C58-B58,"")</f>
         <v>2585</v>
       </c>
+      <c r="L58" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F58), "MISSING", IF(F58&lt;3, "POOR", IF(F58&gt;4.5, "EXCELLENT", IF(AND(F58&gt;=3, F58&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>POOR</v>
+      </c>
+      <c r="M58" s="7" t="str">
+        <f aca="false">IF(L58="UN-CATEGORISED", "AVERAGE", L58)</f>
+        <v>POOR</v>
+      </c>
     </row>
     <row r="59" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="7" t="str">
@@ -7186,6 +7746,14 @@
         <f aca="false">IFERROR(C59-B59,"")</f>
         <v>1000</v>
       </c>
+      <c r="L59" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F59), "MISSING", IF(F59&lt;3, "POOR", IF(F59&gt;4.5, "EXCELLENT", IF(AND(F59&gt;=3, F59&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>POOR</v>
+      </c>
+      <c r="M59" s="7" t="str">
+        <f aca="false">IF(L59="UN-CATEGORISED", "AVERAGE", L59)</f>
+        <v>POOR</v>
+      </c>
     </row>
     <row r="60" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="7" t="str">
@@ -7232,6 +7800,14 @@
         <f aca="false">IFERROR(C60-B60,"")</f>
         <v>317</v>
       </c>
+      <c r="L60" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F60), "MISSING", IF(F60&lt;3, "POOR", IF(F60&gt;4.5, "EXCELLENT", IF(AND(F60&gt;=3, F60&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>AVERAGE</v>
+      </c>
+      <c r="M60" s="7" t="str">
+        <f aca="false">IF(L60="UN-CATEGORISED", "AVERAGE", L60)</f>
+        <v>AVERAGE</v>
+      </c>
     </row>
     <row r="61" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="7" t="str">
@@ -7278,6 +7854,14 @@
         <f aca="false">IFERROR(C61-B61,"")</f>
         <v>850</v>
       </c>
+      <c r="L61" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F61), "MISSING", IF(F61&lt;3, "POOR", IF(F61&gt;4.5, "EXCELLENT", IF(AND(F61&gt;=3, F61&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>EXCELLENT</v>
+      </c>
+      <c r="M61" s="7" t="str">
+        <f aca="false">IF(L61="UN-CATEGORISED", "AVERAGE", L61)</f>
+        <v>EXCELLENT</v>
+      </c>
     </row>
     <row r="62" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="7" t="str">
@@ -7324,6 +7908,14 @@
         <f aca="false">IFERROR(C62-B62,"")</f>
         <v>1200</v>
       </c>
+      <c r="L62" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F62), "MISSING", IF(F62&lt;3, "POOR", IF(F62&gt;4.5, "EXCELLENT", IF(AND(F62&gt;=3, F62&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>EXCELLENT</v>
+      </c>
+      <c r="M62" s="7" t="str">
+        <f aca="false">IF(L62="UN-CATEGORISED", "AVERAGE", L62)</f>
+        <v>EXCELLENT</v>
+      </c>
     </row>
     <row r="63" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="7" t="str">
@@ -7370,6 +7962,14 @@
         <f aca="false">IFERROR(C63-B63,"")</f>
         <v>1200</v>
       </c>
+      <c r="L63" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F63), "MISSING", IF(F63&lt;3, "POOR", IF(F63&gt;4.5, "EXCELLENT", IF(AND(F63&gt;=3, F63&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>EXCELLENT</v>
+      </c>
+      <c r="M63" s="7" t="str">
+        <f aca="false">IF(L63="UN-CATEGORISED", "AVERAGE", L63)</f>
+        <v>EXCELLENT</v>
+      </c>
     </row>
     <row r="64" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="7" t="str">
@@ -7416,6 +8016,14 @@
         <f aca="false">IFERROR(C64-B64,"")</f>
         <v>450</v>
       </c>
+      <c r="L64" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F64), "MISSING", IF(F64&lt;3, "POOR", IF(F64&gt;4.5, "EXCELLENT", IF(AND(F64&gt;=3, F64&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>POOR</v>
+      </c>
+      <c r="M64" s="7" t="str">
+        <f aca="false">IF(L64="UN-CATEGORISED", "AVERAGE", L64)</f>
+        <v>POOR</v>
+      </c>
     </row>
     <row r="65" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="7" t="str">
@@ -7462,6 +8070,14 @@
         <f aca="false">IFERROR(C65-B65,"")</f>
         <v>1946</v>
       </c>
+      <c r="L65" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F65), "MISSING", IF(F65&lt;3, "POOR", IF(F65&gt;4.5, "EXCELLENT", IF(AND(F65&gt;=3, F65&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>EXCELLENT</v>
+      </c>
+      <c r="M65" s="7" t="str">
+        <f aca="false">IF(L65="UN-CATEGORISED", "AVERAGE", L65)</f>
+        <v>EXCELLENT</v>
+      </c>
     </row>
     <row r="66" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="7" t="str">
@@ -7508,6 +8124,14 @@
         <f aca="false">IFERROR(C66-B66,"")</f>
         <v>645</v>
       </c>
+      <c r="L66" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F66), "MISSING", IF(F66&lt;3, "POOR", IF(F66&gt;4.5, "EXCELLENT", IF(AND(F66&gt;=3, F66&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>EXCELLENT</v>
+      </c>
+      <c r="M66" s="7" t="str">
+        <f aca="false">IF(L66="UN-CATEGORISED", "AVERAGE", L66)</f>
+        <v>EXCELLENT</v>
+      </c>
     </row>
     <row r="67" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="7" t="str">
@@ -7554,6 +8178,14 @@
         <f aca="false">IFERROR(C67-B67,"")</f>
         <v>768</v>
       </c>
+      <c r="L67" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F67), "MISSING", IF(F67&lt;3, "POOR", IF(F67&gt;4.5, "EXCELLENT", IF(AND(F67&gt;=3, F67&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>EXCELLENT</v>
+      </c>
+      <c r="M67" s="7" t="str">
+        <f aca="false">IF(L67="UN-CATEGORISED", "AVERAGE", L67)</f>
+        <v>EXCELLENT</v>
+      </c>
     </row>
     <row r="68" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="7" t="str">
@@ -7600,6 +8232,14 @@
         <f aca="false">IFERROR(C68-B68,"")</f>
         <v>940</v>
       </c>
+      <c r="L68" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F68), "MISSING", IF(F68&lt;3, "POOR", IF(F68&gt;4.5, "EXCELLENT", IF(AND(F68&gt;=3, F68&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>AVERAGE</v>
+      </c>
+      <c r="M68" s="7" t="str">
+        <f aca="false">IF(L68="UN-CATEGORISED", "AVERAGE", L68)</f>
+        <v>AVERAGE</v>
+      </c>
     </row>
     <row r="69" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="7" t="str">
@@ -7646,6 +8286,14 @@
         <f aca="false">IFERROR(C69-B69,"")</f>
         <v>941</v>
       </c>
+      <c r="L69" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F69), "MISSING", IF(F69&lt;3, "POOR", IF(F69&gt;4.5, "EXCELLENT", IF(AND(F69&gt;=3, F69&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>EXCELLENT</v>
+      </c>
+      <c r="M69" s="7" t="str">
+        <f aca="false">IF(L69="UN-CATEGORISED", "AVERAGE", L69)</f>
+        <v>EXCELLENT</v>
+      </c>
     </row>
     <row r="70" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="7" t="str">
@@ -7692,6 +8340,14 @@
         <f aca="false">IFERROR(C70-B70,"")</f>
         <v>354</v>
       </c>
+      <c r="L70" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F70), "MISSING", IF(F70&lt;3, "POOR", IF(F70&gt;4.5, "EXCELLENT", IF(AND(F70&gt;=3, F70&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>EXCELLENT</v>
+      </c>
+      <c r="M70" s="7" t="str">
+        <f aca="false">IF(L70="UN-CATEGORISED", "AVERAGE", L70)</f>
+        <v>EXCELLENT</v>
+      </c>
     </row>
     <row r="71" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="7" t="str">
@@ -7738,6 +8394,14 @@
         <f aca="false">IFERROR(C71-B71,"")</f>
         <v>200</v>
       </c>
+      <c r="L71" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F71), "MISSING", IF(F71&lt;3, "POOR", IF(F71&gt;4.5, "EXCELLENT", IF(AND(F71&gt;=3, F71&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>UN-CATEGORISED</v>
+      </c>
+      <c r="M71" s="7" t="str">
+        <f aca="false">IF(L71="UN-CATEGORISED", "AVERAGE", L71)</f>
+        <v>AVERAGE</v>
+      </c>
     </row>
     <row r="72" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="7" t="str">
@@ -7784,6 +8448,14 @@
         <f aca="false">IFERROR(C72-B72,"")</f>
         <v>428</v>
       </c>
+      <c r="L72" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F72), "MISSING", IF(F72&lt;3, "POOR", IF(F72&gt;4.5, "EXCELLENT", IF(AND(F72&gt;=3, F72&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>POOR</v>
+      </c>
+      <c r="M72" s="7" t="str">
+        <f aca="false">IF(L72="UN-CATEGORISED", "AVERAGE", L72)</f>
+        <v>POOR</v>
+      </c>
     </row>
     <row r="73" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="7" t="str">
@@ -7830,6 +8502,14 @@
         <f aca="false">IFERROR(C73-B73,"")</f>
         <v>1001</v>
       </c>
+      <c r="L73" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F73), "MISSING", IF(F73&lt;3, "POOR", IF(F73&gt;4.5, "EXCELLENT", IF(AND(F73&gt;=3, F73&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>EXCELLENT</v>
+      </c>
+      <c r="M73" s="7" t="str">
+        <f aca="false">IF(L73="UN-CATEGORISED", "AVERAGE", L73)</f>
+        <v>EXCELLENT</v>
+      </c>
     </row>
     <row r="74" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="7" t="str">
@@ -7876,6 +8556,14 @@
         <f aca="false">IFERROR(C74-B74,"")</f>
         <v>134</v>
       </c>
+      <c r="L74" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F74), "MISSING", IF(F74&lt;3, "POOR", IF(F74&gt;4.5, "EXCELLENT", IF(AND(F74&gt;=3, F74&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>EXCELLENT</v>
+      </c>
+      <c r="M74" s="7" t="str">
+        <f aca="false">IF(L74="UN-CATEGORISED", "AVERAGE", L74)</f>
+        <v>EXCELLENT</v>
+      </c>
     </row>
     <row r="75" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="7" t="str">
@@ -7922,6 +8610,14 @@
         <f aca="false">IFERROR(C75-B75,"")</f>
         <v>1880</v>
       </c>
+      <c r="L75" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F75), "MISSING", IF(F75&lt;3, "POOR", IF(F75&gt;4.5, "EXCELLENT", IF(AND(F75&gt;=3, F75&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>EXCELLENT</v>
+      </c>
+      <c r="M75" s="7" t="str">
+        <f aca="false">IF(L75="UN-CATEGORISED", "AVERAGE", L75)</f>
+        <v>EXCELLENT</v>
+      </c>
     </row>
     <row r="76" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="7" t="str">
@@ -7968,6 +8664,14 @@
         <f aca="false">IFERROR(C76-B76,"")</f>
         <v>227</v>
       </c>
+      <c r="L76" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F76), "MISSING", IF(F76&lt;3, "POOR", IF(F76&gt;4.5, "EXCELLENT", IF(AND(F76&gt;=3, F76&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>EXCELLENT</v>
+      </c>
+      <c r="M76" s="7" t="str">
+        <f aca="false">IF(L76="UN-CATEGORISED", "AVERAGE", L76)</f>
+        <v>EXCELLENT</v>
+      </c>
     </row>
     <row r="77" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="7" t="str">
@@ -8014,6 +8718,14 @@
         <f aca="false">IFERROR(C77-B77,"")</f>
         <v>800</v>
       </c>
+      <c r="L77" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F77), "MISSING", IF(F77&lt;3, "POOR", IF(F77&gt;4.5, "EXCELLENT", IF(AND(F77&gt;=3, F77&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>EXCELLENT</v>
+      </c>
+      <c r="M77" s="7" t="str">
+        <f aca="false">IF(L77="UN-CATEGORISED", "AVERAGE", L77)</f>
+        <v>EXCELLENT</v>
+      </c>
     </row>
     <row r="78" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="7" t="str">
@@ -8060,6 +8772,14 @@
         <f aca="false">IFERROR(C78-B78,"")</f>
         <v>85</v>
       </c>
+      <c r="L78" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F78), "MISSING", IF(F78&lt;3, "POOR", IF(F78&gt;4.5, "EXCELLENT", IF(AND(F78&gt;=3, F78&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>EXCELLENT</v>
+      </c>
+      <c r="M78" s="7" t="str">
+        <f aca="false">IF(L78="UN-CATEGORISED", "AVERAGE", L78)</f>
+        <v>EXCELLENT</v>
+      </c>
     </row>
     <row r="79" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="7" t="str">
@@ -8106,6 +8826,14 @@
         <f aca="false">IFERROR(C79-B79,"")</f>
         <v>153</v>
       </c>
+      <c r="L79" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F79), "MISSING", IF(F79&lt;3, "POOR", IF(F79&gt;4.5, "EXCELLENT", IF(AND(F79&gt;=3, F79&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>EXCELLENT</v>
+      </c>
+      <c r="M79" s="7" t="str">
+        <f aca="false">IF(L79="UN-CATEGORISED", "AVERAGE", L79)</f>
+        <v>EXCELLENT</v>
+      </c>
     </row>
     <row r="80" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="7" t="str">
@@ -8152,6 +8880,14 @@
         <f aca="false">IFERROR(C80-B80,"")</f>
         <v>616</v>
       </c>
+      <c r="L80" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F80), "MISSING", IF(F80&lt;3, "POOR", IF(F80&gt;4.5, "EXCELLENT", IF(AND(F80&gt;=3, F80&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>EXCELLENT</v>
+      </c>
+      <c r="M80" s="7" t="str">
+        <f aca="false">IF(L80="UN-CATEGORISED", "AVERAGE", L80)</f>
+        <v>EXCELLENT</v>
+      </c>
     </row>
     <row r="81" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="7" t="str">
@@ -8198,6 +8934,14 @@
         <f aca="false">IFERROR(C81-B81,"")</f>
         <v>640</v>
       </c>
+      <c r="L81" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F81), "MISSING", IF(F81&lt;3, "POOR", IF(F81&gt;4.5, "EXCELLENT", IF(AND(F81&gt;=3, F81&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>AVERAGE</v>
+      </c>
+      <c r="M81" s="7" t="str">
+        <f aca="false">IF(L81="UN-CATEGORISED", "AVERAGE", L81)</f>
+        <v>AVERAGE</v>
+      </c>
     </row>
     <row r="82" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="7" t="str">
@@ -8244,6 +8988,14 @@
         <f aca="false">IFERROR(C82-B82,"")</f>
         <v>301</v>
       </c>
+      <c r="L82" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F82), "MISSING", IF(F82&lt;3, "POOR", IF(F82&gt;4.5, "EXCELLENT", IF(AND(F82&gt;=3, F82&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>EXCELLENT</v>
+      </c>
+      <c r="M82" s="7" t="str">
+        <f aca="false">IF(L82="UN-CATEGORISED", "AVERAGE", L82)</f>
+        <v>EXCELLENT</v>
+      </c>
     </row>
     <row r="83" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="7" t="str">
@@ -8290,6 +9042,14 @@
         <f aca="false">IFERROR(C83-B83,"")</f>
         <v>640</v>
       </c>
+      <c r="L83" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F83), "MISSING", IF(F83&lt;3, "POOR", IF(F83&gt;4.5, "EXCELLENT", IF(AND(F83&gt;=3, F83&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>AVERAGE</v>
+      </c>
+      <c r="M83" s="7" t="str">
+        <f aca="false">IF(L83="UN-CATEGORISED", "AVERAGE", L83)</f>
+        <v>AVERAGE</v>
+      </c>
     </row>
     <row r="84" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="7" t="str">
@@ -8336,6 +9096,14 @@
         <f aca="false">IFERROR(C84-B84,"")</f>
         <v>151</v>
       </c>
+      <c r="L84" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F84), "MISSING", IF(F84&lt;3, "POOR", IF(F84&gt;4.5, "EXCELLENT", IF(AND(F84&gt;=3, F84&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>EXCELLENT</v>
+      </c>
+      <c r="M84" s="7" t="str">
+        <f aca="false">IF(L84="UN-CATEGORISED", "AVERAGE", L84)</f>
+        <v>EXCELLENT</v>
+      </c>
     </row>
     <row r="85" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="7" t="str">
@@ -8382,6 +9150,14 @@
         <f aca="false">IFERROR(C85-B85,"")</f>
         <v>330</v>
       </c>
+      <c r="L85" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F85), "MISSING", IF(F85&lt;3, "POOR", IF(F85&gt;4.5, "EXCELLENT", IF(AND(F85&gt;=3, F85&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>POOR</v>
+      </c>
+      <c r="M85" s="7" t="str">
+        <f aca="false">IF(L85="UN-CATEGORISED", "AVERAGE", L85)</f>
+        <v>POOR</v>
+      </c>
     </row>
     <row r="86" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="7" t="str">
@@ -8428,6 +9204,14 @@
         <f aca="false">IFERROR(C86-B86,"")</f>
         <v>355</v>
       </c>
+      <c r="L86" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F86), "MISSING", IF(F86&lt;3, "POOR", IF(F86&gt;4.5, "EXCELLENT", IF(AND(F86&gt;=3, F86&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>POOR</v>
+      </c>
+      <c r="M86" s="7" t="str">
+        <f aca="false">IF(L86="UN-CATEGORISED", "AVERAGE", L86)</f>
+        <v>POOR</v>
+      </c>
     </row>
     <row r="87" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="7" t="str">
@@ -8474,6 +9258,14 @@
         <f aca="false">IFERROR(C87-B87,"")</f>
         <v>101</v>
       </c>
+      <c r="L87" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F87), "MISSING", IF(F87&lt;3, "POOR", IF(F87&gt;4.5, "EXCELLENT", IF(AND(F87&gt;=3, F87&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>EXCELLENT</v>
+      </c>
+      <c r="M87" s="7" t="str">
+        <f aca="false">IF(L87="UN-CATEGORISED", "AVERAGE", L87)</f>
+        <v>EXCELLENT</v>
+      </c>
     </row>
     <row r="88" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="7" t="str">
@@ -8520,6 +9312,14 @@
         <f aca="false">IFERROR(C88-B88,"")</f>
         <v>510</v>
       </c>
+      <c r="L88" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F88), "MISSING", IF(F88&lt;3, "POOR", IF(F88&gt;4.5, "EXCELLENT", IF(AND(F88&gt;=3, F88&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>EXCELLENT</v>
+      </c>
+      <c r="M88" s="7" t="str">
+        <f aca="false">IF(L88="UN-CATEGORISED", "AVERAGE", L88)</f>
+        <v>EXCELLENT</v>
+      </c>
     </row>
     <row r="89" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="7" t="str">
@@ -8566,6 +9366,14 @@
         <f aca="false">IFERROR(C89-B89,"")</f>
         <v>968</v>
       </c>
+      <c r="L89" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F89), "MISSING", IF(F89&lt;3, "POOR", IF(F89&gt;4.5, "EXCELLENT", IF(AND(F89&gt;=3, F89&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>EXCELLENT</v>
+      </c>
+      <c r="M89" s="7" t="str">
+        <f aca="false">IF(L89="UN-CATEGORISED", "AVERAGE", L89)</f>
+        <v>EXCELLENT</v>
+      </c>
     </row>
     <row r="90" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="7" t="str">
@@ -8612,6 +9420,14 @@
         <f aca="false">IFERROR(C90-B90,"")</f>
         <v>1360</v>
       </c>
+      <c r="L90" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F90), "MISSING", IF(F90&lt;3, "POOR", IF(F90&gt;4.5, "EXCELLENT", IF(AND(F90&gt;=3, F90&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>EXCELLENT</v>
+      </c>
+      <c r="M90" s="7" t="str">
+        <f aca="false">IF(L90="UN-CATEGORISED", "AVERAGE", L90)</f>
+        <v>EXCELLENT</v>
+      </c>
     </row>
     <row r="91" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="7" t="str">
@@ -8658,6 +9474,14 @@
         <f aca="false">IFERROR(C91-B91,"")</f>
         <v>830</v>
       </c>
+      <c r="L91" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F91), "MISSING", IF(F91&lt;3, "POOR", IF(F91&gt;4.5, "EXCELLENT", IF(AND(F91&gt;=3, F91&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>EXCELLENT</v>
+      </c>
+      <c r="M91" s="7" t="str">
+        <f aca="false">IF(L91="UN-CATEGORISED", "AVERAGE", L91)</f>
+        <v>EXCELLENT</v>
+      </c>
     </row>
     <row r="92" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="7" t="str">
@@ -8704,6 +9528,14 @@
         <f aca="false">IFERROR(C92-B92,"")</f>
         <v>472</v>
       </c>
+      <c r="L92" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F92), "MISSING", IF(F92&lt;3, "POOR", IF(F92&gt;4.5, "EXCELLENT", IF(AND(F92&gt;=3, F92&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>UN-CATEGORISED</v>
+      </c>
+      <c r="M92" s="7" t="str">
+        <f aca="false">IF(L92="UN-CATEGORISED", "AVERAGE", L92)</f>
+        <v>AVERAGE</v>
+      </c>
     </row>
     <row r="93" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="7" t="str">
@@ -8750,6 +9582,14 @@
         <f aca="false">IFERROR(C93-B93,"")</f>
         <v>620</v>
       </c>
+      <c r="L93" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F93), "MISSING", IF(F93&lt;3, "POOR", IF(F93&gt;4.5, "EXCELLENT", IF(AND(F93&gt;=3, F93&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>EXCELLENT</v>
+      </c>
+      <c r="M93" s="7" t="str">
+        <f aca="false">IF(L93="UN-CATEGORISED", "AVERAGE", L93)</f>
+        <v>EXCELLENT</v>
+      </c>
     </row>
     <row r="94" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="7" t="str">
@@ -8796,6 +9636,14 @@
         <f aca="false">IFERROR(C94-B94,"")</f>
         <v>500</v>
       </c>
+      <c r="L94" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F94), "MISSING", IF(F94&lt;3, "POOR", IF(F94&gt;4.5, "EXCELLENT", IF(AND(F94&gt;=3, F94&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>UN-CATEGORISED</v>
+      </c>
+      <c r="M94" s="7" t="str">
+        <f aca="false">IF(L94="UN-CATEGORISED", "AVERAGE", L94)</f>
+        <v>AVERAGE</v>
+      </c>
     </row>
     <row r="95" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="7" t="str">
@@ -8842,6 +9690,14 @@
         <f aca="false">IFERROR(C95-B95,"")</f>
         <v>24</v>
       </c>
+      <c r="L95" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F95), "MISSING", IF(F95&lt;3, "POOR", IF(F95&gt;4.5, "EXCELLENT", IF(AND(F95&gt;=3, F95&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>EXCELLENT</v>
+      </c>
+      <c r="M95" s="7" t="str">
+        <f aca="false">IF(L95="UN-CATEGORISED", "AVERAGE", L95)</f>
+        <v>EXCELLENT</v>
+      </c>
     </row>
     <row r="96" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="7" t="str">
@@ -8888,6 +9744,14 @@
         <f aca="false">IFERROR(C96-B96,"")</f>
         <v>39</v>
       </c>
+      <c r="L96" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F96), "MISSING", IF(F96&lt;3, "POOR", IF(F96&gt;4.5, "EXCELLENT", IF(AND(F96&gt;=3, F96&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>EXCELLENT</v>
+      </c>
+      <c r="M96" s="7" t="str">
+        <f aca="false">IF(L96="UN-CATEGORISED", "AVERAGE", L96)</f>
+        <v>EXCELLENT</v>
+      </c>
     </row>
     <row r="97" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="7" t="str">
@@ -8934,6 +9798,14 @@
         <f aca="false">IFERROR(C97-B97,"")</f>
         <v>1000</v>
       </c>
+      <c r="L97" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F97), "MISSING", IF(F97&lt;3, "POOR", IF(F97&gt;4.5, "EXCELLENT", IF(AND(F97&gt;=3, F97&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>EXCELLENT</v>
+      </c>
+      <c r="M97" s="7" t="str">
+        <f aca="false">IF(L97="UN-CATEGORISED", "AVERAGE", L97)</f>
+        <v>EXCELLENT</v>
+      </c>
     </row>
     <row r="98" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="7" t="str">
@@ -8980,6 +9852,14 @@
         <f aca="false">IFERROR(C98-B98,"")</f>
         <v>595</v>
       </c>
+      <c r="L98" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F98), "MISSING", IF(F98&lt;3, "POOR", IF(F98&gt;4.5, "EXCELLENT", IF(AND(F98&gt;=3, F98&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>EXCELLENT</v>
+      </c>
+      <c r="M98" s="7" t="str">
+        <f aca="false">IF(L98="UN-CATEGORISED", "AVERAGE", L98)</f>
+        <v>EXCELLENT</v>
+      </c>
     </row>
     <row r="99" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="7" t="str">
@@ -9026,6 +9906,14 @@
         <f aca="false">IFERROR(C99-B99,"")</f>
         <v>1329</v>
       </c>
+      <c r="L99" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F99), "MISSING", IF(F99&lt;3, "POOR", IF(F99&gt;4.5, "EXCELLENT", IF(AND(F99&gt;=3, F99&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>AVERAGE</v>
+      </c>
+      <c r="M99" s="7" t="str">
+        <f aca="false">IF(L99="UN-CATEGORISED", "AVERAGE", L99)</f>
+        <v>AVERAGE</v>
+      </c>
     </row>
     <row r="100" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="7" t="str">
@@ -9072,6 +9960,14 @@
         <f aca="false">IFERROR(C100-B100,"")</f>
         <v>794</v>
       </c>
+      <c r="L100" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F100), "MISSING", IF(F100&lt;3, "POOR", IF(F100&gt;4.5, "EXCELLENT", IF(AND(F100&gt;=3, F100&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>EXCELLENT</v>
+      </c>
+      <c r="M100" s="7" t="str">
+        <f aca="false">IF(L100="UN-CATEGORISED", "AVERAGE", L100)</f>
+        <v>EXCELLENT</v>
+      </c>
     </row>
     <row r="101" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="7" t="str">
@@ -9118,6 +10014,14 @@
         <f aca="false">IFERROR(C101-B101,"")</f>
         <v>390</v>
       </c>
+      <c r="L101" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F101), "MISSING", IF(F101&lt;3, "POOR", IF(F101&gt;4.5, "EXCELLENT", IF(AND(F101&gt;=3, F101&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>AVERAGE</v>
+      </c>
+      <c r="M101" s="7" t="str">
+        <f aca="false">IF(L101="UN-CATEGORISED", "AVERAGE", L101)</f>
+        <v>AVERAGE</v>
+      </c>
     </row>
     <row r="102" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="7" t="str">
@@ -9164,6 +10068,14 @@
         <f aca="false">IFERROR(C102-B102,"")</f>
         <v>41</v>
       </c>
+      <c r="L102" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F102), "MISSING", IF(F102&lt;3, "POOR", IF(F102&gt;4.5, "EXCELLENT", IF(AND(F102&gt;=3, F102&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>EXCELLENT</v>
+      </c>
+      <c r="M102" s="7" t="str">
+        <f aca="false">IF(L102="UN-CATEGORISED", "AVERAGE", L102)</f>
+        <v>EXCELLENT</v>
+      </c>
     </row>
     <row r="103" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="7" t="str">
@@ -9210,6 +10122,14 @@
         <f aca="false">IFERROR(C103-B103,"")</f>
         <v>824</v>
       </c>
+      <c r="L103" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F103), "MISSING", IF(F103&lt;3, "POOR", IF(F103&gt;4.5, "EXCELLENT", IF(AND(F103&gt;=3, F103&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>POOR</v>
+      </c>
+      <c r="M103" s="7" t="str">
+        <f aca="false">IF(L103="UN-CATEGORISED", "AVERAGE", L103)</f>
+        <v>POOR</v>
+      </c>
     </row>
     <row r="104" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="7" t="str">
@@ -9256,6 +10176,14 @@
         <f aca="false">IFERROR(C104-B104,"")</f>
         <v>318</v>
       </c>
+      <c r="L104" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F104), "MISSING", IF(F104&lt;3, "POOR", IF(F104&gt;4.5, "EXCELLENT", IF(AND(F104&gt;=3, F104&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>POOR</v>
+      </c>
+      <c r="M104" s="7" t="str">
+        <f aca="false">IF(L104="UN-CATEGORISED", "AVERAGE", L104)</f>
+        <v>POOR</v>
+      </c>
     </row>
     <row r="105" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="7" t="str">
@@ -9302,6 +10230,14 @@
         <f aca="false">IFERROR(C105-B105,"")</f>
         <v>450</v>
       </c>
+      <c r="L105" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F105), "MISSING", IF(F105&lt;3, "POOR", IF(F105&gt;4.5, "EXCELLENT", IF(AND(F105&gt;=3, F105&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>EXCELLENT</v>
+      </c>
+      <c r="M105" s="7" t="str">
+        <f aca="false">IF(L105="UN-CATEGORISED", "AVERAGE", L105)</f>
+        <v>EXCELLENT</v>
+      </c>
     </row>
     <row r="106" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="7" t="str">
@@ -9348,6 +10284,14 @@
         <f aca="false">IFERROR(C106-B106,"")</f>
         <v>352</v>
       </c>
+      <c r="L106" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F106), "MISSING", IF(F106&lt;3, "POOR", IF(F106&gt;4.5, "EXCELLENT", IF(AND(F106&gt;=3, F106&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>EXCELLENT</v>
+      </c>
+      <c r="M106" s="7" t="str">
+        <f aca="false">IF(L106="UN-CATEGORISED", "AVERAGE", L106)</f>
+        <v>EXCELLENT</v>
+      </c>
     </row>
     <row r="107" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="7" t="str">
@@ -9394,6 +10338,14 @@
         <f aca="false">IFERROR(C107-B107,"")</f>
         <v>750</v>
       </c>
+      <c r="L107" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F107), "MISSING", IF(F107&lt;3, "POOR", IF(F107&gt;4.5, "EXCELLENT", IF(AND(F107&gt;=3, F107&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>EXCELLENT</v>
+      </c>
+      <c r="M107" s="7" t="str">
+        <f aca="false">IF(L107="UN-CATEGORISED", "AVERAGE", L107)</f>
+        <v>EXCELLENT</v>
+      </c>
     </row>
     <row r="108" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="7" t="str">
@@ -9440,6 +10392,14 @@
         <f aca="false">IFERROR(C108-B108,"")</f>
         <v>1418</v>
       </c>
+      <c r="L108" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F108), "MISSING", IF(F108&lt;3, "POOR", IF(F108&gt;4.5, "EXCELLENT", IF(AND(F108&gt;=3, F108&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>POOR</v>
+      </c>
+      <c r="M108" s="7" t="str">
+        <f aca="false">IF(L108="UN-CATEGORISED", "AVERAGE", L108)</f>
+        <v>POOR</v>
+      </c>
     </row>
     <row r="109" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="7" t="str">
@@ -9486,6 +10446,14 @@
         <f aca="false">IFERROR(C109-B109,"")</f>
         <v>592</v>
       </c>
+      <c r="L109" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F109), "MISSING", IF(F109&lt;3, "POOR", IF(F109&gt;4.5, "EXCELLENT", IF(AND(F109&gt;=3, F109&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>AVERAGE</v>
+      </c>
+      <c r="M109" s="7" t="str">
+        <f aca="false">IF(L109="UN-CATEGORISED", "AVERAGE", L109)</f>
+        <v>AVERAGE</v>
+      </c>
     </row>
     <row r="110" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="7" t="str">
@@ -9532,6 +10500,14 @@
         <f aca="false">IFERROR(C110-B110,"")</f>
         <v>497</v>
       </c>
+      <c r="L110" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F110), "MISSING", IF(F110&lt;3, "POOR", IF(F110&gt;4.5, "EXCELLENT", IF(AND(F110&gt;=3, F110&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>EXCELLENT</v>
+      </c>
+      <c r="M110" s="7" t="str">
+        <f aca="false">IF(L110="UN-CATEGORISED", "AVERAGE", L110)</f>
+        <v>EXCELLENT</v>
+      </c>
     </row>
     <row r="111" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A111" s="7" t="str">
@@ -9578,6 +10554,14 @@
         <f aca="false">IFERROR(C111-B111,"")</f>
         <v>37</v>
       </c>
+      <c r="L111" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F111), "MISSING", IF(F111&lt;3, "POOR", IF(F111&gt;4.5, "EXCELLENT", IF(AND(F111&gt;=3, F111&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>EXCELLENT</v>
+      </c>
+      <c r="M111" s="7" t="str">
+        <f aca="false">IF(L111="UN-CATEGORISED", "AVERAGE", L111)</f>
+        <v>EXCELLENT</v>
+      </c>
     </row>
     <row r="112" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A112" s="7" t="str">
@@ -9624,6 +10608,14 @@
         <f aca="false">IFERROR(C112-B112,"")</f>
         <v>2452</v>
       </c>
+      <c r="L112" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F112), "MISSING", IF(F112&lt;3, "POOR", IF(F112&gt;4.5, "EXCELLENT", IF(AND(F112&gt;=3, F112&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>UN-CATEGORISED</v>
+      </c>
+      <c r="M112" s="7" t="str">
+        <f aca="false">IF(L112="UN-CATEGORISED", "AVERAGE", L112)</f>
+        <v>AVERAGE</v>
+      </c>
     </row>
     <row r="113" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A113" s="7" t="str">
@@ -9670,6 +10662,14 @@
         <f aca="false">IFERROR(C113-B113,"")</f>
         <v>1721</v>
       </c>
+      <c r="L113" s="7" t="str">
+        <f aca="false">IF(ISBLANK(F113), "MISSING", IF(F113&lt;3, "POOR", IF(F113&gt;4.5, "EXCELLENT", IF(AND(F113&gt;=3, F113&lt;=4), "AVERAGE", "UN-CATEGORISED"))))</f>
+        <v>EXCELLENT</v>
+      </c>
+      <c r="M113" s="7" t="str">
+        <f aca="false">IF(L113="UN-CATEGORISED", "AVERAGE", L113)</f>
+        <v>EXCELLENT</v>
+      </c>
     </row>
     <row r="114" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A114" s="7" t="str">
@@ -9681,10 +10681,24 @@
       <c r="G116" s="24"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G114"/>
+  <autoFilter ref="A1:L114"/>
   <conditionalFormatting sqref="H2:J113">
-    <cfRule type="containsText" priority="2" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="ok" dxfId="8">
+    <cfRule type="containsText" priority="2" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="ok" dxfId="11">
       <formula>NOT(ISERROR(SEARCH("ok",H2)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L2:M113">
+    <cfRule type="containsText" priority="3" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="UN-CATEGORISED" dxfId="12">
+      <formula>NOT(ISERROR(SEARCH("UN-CATEGORISED",L2)))</formula>
+    </cfRule>
+    <cfRule type="containsText" priority="4" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="EXCELLENT" dxfId="11">
+      <formula>NOT(ISERROR(SEARCH("EXCELLENT",L2)))</formula>
+    </cfRule>
+    <cfRule type="containsText" priority="5" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="POOR" dxfId="13">
+      <formula>NOT(ISERROR(SEARCH("POOR",L2)))</formula>
+    </cfRule>
+    <cfRule type="containsText" priority="6" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="AVERAGE" dxfId="14">
+      <formula>NOT(ISERROR(SEARCH("AVERAGE",L2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>